<commit_message>
Update H01 and H12 price years in the workbook
Only cells Ledger!Q2 and Ledger!Q13 changed; every other part of the
file is byte-identical. The workbook matches ledger.json again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -3733,7 +3733,7 @@
         <v>70</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>71</v>
+        <v>335</v>
       </c>
       <c r="R2" s="10" t="s">
         <v>72</v>
@@ -4345,7 +4345,7 @@
         <v>81</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>193</v>
+        <v>256</v>
       </c>
       <c r="R13" s="10" t="s">
         <v>194</v>

</xml_diff>

<commit_message>
Check every rebased price year against its source; correct I05
ledger.json and workbook (approved by Stan Gilmour): I05 year 2012/13
-> 2013, as stated in the source. rebase.json (still draft): leave out
H23, H35 and H36 (no stated price base) and H28 (mixed base); notes on
each remaining entry quote its source. 20 entries remain.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -5972,8 +5972,10 @@
       <c r="P42" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="Q42" s="10" t="s">
-        <v>454</v>
+      <c r="Q42" s="10" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
       </c>
       <c r="R42" s="10" t="s">
         <v>455</v>

</xml_diff>

<commit_message>
Resolve the data queries
Approved by Stan Gilmour, 25 September 2026 (see DATA-QUERIES.md and
CHANGELOG.md): I17 revised from YEF's formal pre-court diversion strand;
H29 and H30 headlines use source figures; H19 and I07 wording matches
their sources; I02 source names its author; P01 note on the 2026 Green
Book; four URLs updated. Calculator notes for mixed ranges and derived
ratios, and 'Benefit not established' for I09 (site text). Workbook
updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -4126,8 +4126,10 @@
       <c r="R9" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="S9" s="11" t="s">
-        <v>150</v>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1016/S2468-2667(21)00232-2</t>
+        </is>
       </c>
       <c r="T9" s="10" t="s">
         <v>151</v>
@@ -4716,8 +4718,10 @@
       <c r="H20" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="I20" s="10" t="s">
-        <v>253</v>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spend per child per year</t>
+        </is>
       </c>
       <c r="J20" s="10" t="s">
         <v>254</v>
@@ -4743,8 +4747,10 @@
       <c r="S20" s="11" t="s">
         <v>258</v>
       </c>
-      <c r="T20" s="10" t="s">
-        <v>259</v>
+      <c r="T20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CMA (2022) found the largest providers earn materially higher profits than a working market would. NAO figure is spend per child; its residential category includes secure units, residential care homes and residential schools.</t>
+        </is>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5791,11 +5797,15 @@
       <c r="Q39" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="R39" s="10" t="s">
-        <v>424</v>
-      </c>
-      <c r="S39" s="11" t="s">
-        <v>425</v>
+      <c r="R39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ullah et al. (2025), Lancet Psychiatry (ROSHNI-2 economic evaluation)</t>
+        </is>
+      </c>
+      <c r="S39" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1016/S2215-0366(25)00039-2</t>
+        </is>
       </c>
       <c r="T39" s="10" t="s">
         <v>426</v>
@@ -6077,8 +6087,10 @@
       <c r="I44" s="10" t="s">
         <v>471</v>
       </c>
-      <c r="J44" s="10" t="s">
-        <v>472</v>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">£1,177 per participant; public-sector savings 2.8–6.1 times cost; societal savings £16,435 over 25 years; payback 5–8 years</t>
+        </is>
       </c>
       <c r="K44" s="10" t="s">
         <v>473</v>
@@ -6685,17 +6697,25 @@
       <c r="G54" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="H54" s="10" t="s">
-        <v>558</v>
-      </c>
-      <c r="I54" s="10" t="s">
-        <v>559</v>
-      </c>
-      <c r="J54" s="10" t="s">
-        <v>560</v>
-      </c>
-      <c r="K54" s="10" t="s">
-        <v>518</v>
+      <c r="H54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formal pre-court diversion</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effect on reoffending and violence</t>
+        </is>
+      </c>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">−14% reoffending (moderate confidence, 35 studies); −25% violence (low confidence, 5 studies); UK average cost £1,426 per child</t>
+        </is>
+      </c>
+      <c r="K54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective, cost unclear</t>
+        </is>
       </c>
       <c r="L54" s="10" t="s">
         <v>561</v>
@@ -6709,19 +6729,31 @@
       <c r="O54" s="10" t="s">
         <v>520</v>
       </c>
-      <c r="P54" s="10" t="s">
-        <v>563</v>
-      </c>
-      <c r="Q54" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="R54" s="10" t="s">
-        <v>564</v>
-      </c>
-      <c r="S54" s="11" t="s">
-        <v>565</v>
-      </c>
-      <c r="T54" s="10"/>
+      <c r="P54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mostly North America and Australia; UK costs</t>
+        </is>
+      </c>
+      <c r="Q54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">not stated</t>
+        </is>
+      </c>
+      <c r="R54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Youth Endowment Fund Toolkit, Formal pre-court diversion</t>
+        </is>
+      </c>
+      <c r="S54" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://youthendowmentfund.org.uk/toolkit/formal-pre-court-diversion/</t>
+        </is>
+      </c>
+      <c r="T54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Replaces YEF's earlier pre-court diversion strand (−13% reoffending, high confidence, low cost). Informal pre-court diversion is now a separate strand.</t>
+        </is>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
@@ -7869,8 +7901,10 @@
       <c r="S73" s="11" t="s">
         <v>753</v>
       </c>
-      <c r="T73" s="10" t="s">
-        <v>754</v>
+      <c r="T73" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health.</t>
+        </is>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8230,8 +8264,10 @@
       <c r="R80" s="10" t="s">
         <v>808</v>
       </c>
-      <c r="S80" s="11" t="s">
-        <v>809</v>
+      <c r="S80" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
+        </is>
       </c>
       <c r="T80" s="10"/>
     </row>
@@ -8282,8 +8318,10 @@
       <c r="R81" s="10" t="s">
         <v>813</v>
       </c>
-      <c r="S81" s="11" t="s">
-        <v>814</v>
+      <c r="S81" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+        </is>
       </c>
       <c r="T81" s="10"/>
     </row>
@@ -8671,7 +8709,7 @@
     <hyperlink ref="S6" r:id="rId5" display="https://doi.org/10.1111/acer.14705"/>
     <hyperlink ref="S7" r:id="rId6" display="http://wrap.warwick.ac.uk/37026/"/>
     <hyperlink ref="S8" r:id="rId7" display="https://pubmed.ncbi.nlm.nih.gov/40168916/"/>
-    <hyperlink ref="S9" r:id="rId8" display="https://www.sciencedirect.com/science/article/pii/S2468266721002322"/>
+    <hyperlink ref="S9" r:id="rId8" display="https://doi.org/10.1016/S2468-2667(21)00232-2"/>
     <hyperlink ref="S10" r:id="rId9" display="https://doi.org/10.1111/jcpp.12573"/>
     <hyperlink ref="S11" r:id="rId10" display="https://pubmed.ncbi.nlm.nih.gov/11473907/"/>
     <hyperlink ref="S12" r:id="rId11" display="https://doi.org/10.1016/j.socscimed.2018.05.014"/>
@@ -8701,7 +8739,7 @@
     <hyperlink ref="S36" r:id="rId35" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
     <hyperlink ref="S37" r:id="rId36" display="https://www.economicsobservatory.com/youth-violence-in-england-and-wales-what-can-be-done"/>
     <hyperlink ref="S38" r:id="rId37" display="https://doi.org/10.1017/S0033291718001940"/>
-    <hyperlink ref="S39" r:id="rId38" display="https://www.sciencedirect.com/science/article/pii/S2215036625000392"/>
+    <hyperlink ref="S39" r:id="rId38" display="https://doi.org/10.1016/S2215-0366(25)00039-2"/>
     <hyperlink ref="S40" r:id="rId39" display="https://doi.org/10.1111/add.13160"/>
     <hyperlink ref="S41" r:id="rId40" display="https://doi.org/10.1111/add.16176"/>
     <hyperlink ref="S42" r:id="rId41" display="https://doi.org/10.1111/jep.12799"/>
@@ -8716,7 +8754,7 @@
     <hyperlink ref="S51" r:id="rId50" display="https://youthendowmentfund.org.uk/toolkit/mentoring/"/>
     <hyperlink ref="S52" r:id="rId51" display="https://youthendowmentfund.org.uk/toolkit/focused-deterrence/"/>
     <hyperlink ref="S53" r:id="rId52" display="https://youthendowmentfund.org.uk/toolkit/trauma-specific-therapies/"/>
-    <hyperlink ref="S54" r:id="rId53" display="https://youthendowmentfund.org.uk/toolkit/pre-court-diversion/"/>
+    <hyperlink ref="S54" r:id="rId53" display="https://youthendowmentfund.org.uk/toolkit/formal-pre-court-diversion/"/>
     <hyperlink ref="S55" r:id="rId54" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC6697182/"/>
     <hyperlink ref="S56" r:id="rId55" display="https://doi.org/10.1111/jcpp.12743"/>
     <hyperlink ref="S57" r:id="rId56" display="https://www.gov.uk/government/publications/violence-reduction-units-year-ending-march-2023-evaluation-report/violence-reduction-units-2022-to-2023"/>
@@ -8742,8 +8780,8 @@
     <hyperlink ref="S77" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
     <hyperlink ref="S78" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
     <hyperlink ref="S79" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
-    <hyperlink ref="S80" r:id="rId79" display="https://www.health.org.uk/publications/health-in-2040"/>
-    <hyperlink ref="S81" r:id="rId80" display="https://www.health.org.uk/press-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by"/>
+    <hyperlink ref="S80" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
+    <hyperlink ref="S81" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
     <hyperlink ref="S82" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
     <hyperlink ref="S83" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
     <hyperlink ref="S84" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>

</xml_diff>

<commit_message>
Correct H18, H22, H23, H28, H35 and H36 from their primary sources
Six Priority 1 sources read in full and checked against their entries.
Approved by Stan Gilmour KPM FRSA on 27 September 2026. The same cells
are updated in the workbook, and every Ledger-sheet field matches
ledger.json. The H36 rebase is held; see DATA-QUERIES.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="940">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -763,7 +763,7 @@
     <t xml:space="preserve">Annual cost to the economy</t>
   </si>
   <si>
-    <t xml:space="preserve">£43bn: NHS and social care £20bn; productivity £21.5bn; justice and education £1.5bn; benefits £1.9bn</t>
+    <t>£43bn: NHS and social care £20bn; productivity £21.5bn; justice and education £1.5bn; plus benefits £1.9bn, outside the total (transfers)</t>
   </si>
   <si>
     <t xml:space="preserve">Charity-commissioned model</t>
@@ -778,7 +778,7 @@
     <t xml:space="preserve">https://ukabif.org.uk/news/701354/Hidden-toll-of-brain-injury-costs-economy-43-billion-a-year-.htm</t>
   </si>
   <si>
-    <t xml:space="preserve">Wellbeing loss of £91.5bn a year reported separately (secondary summary). Includes stroke and tumours, not only TBI.</t>
+    <t>Covers traumatic brain injury, stroke and brain tumour, about 85% of ABI episodes; other causes are not costed (p.9). The report calls the total both the lifetime costs of ABI in 2023/24 (p.9) and a typical year (p.25). Price bases are mixed. Wellbeing loss of £91.5bn a year reported separately (pp.5, 7).</t>
   </si>
   <si>
     <t xml:space="preserve">H19</t>
@@ -898,7 +898,7 @@
     <t xml:space="preserve">https://www.ias.org.uk/factsheet/economy/</t>
   </si>
   <si>
-    <t xml:space="preserve">Contested: critics argue little falls directly on taxpayers and that this is a cost, not cost-benefit, analysis.</t>
+    <t>Data year 2021/22; price base not stated for all components (methodology, pp.1–2). Contested: critics argue little falls directly on taxpayers and that this is a cost, not cost-benefit, analysis.</t>
   </si>
   <si>
     <t xml:space="preserve">H23</t>
@@ -925,7 +925,7 @@
     <t xml:space="preserve">https://assets.publishing.service.gov.uk/media/60eef5588fa8f50c768386fd/independent-review-of-drugs-part-2-annexes.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">Spend on treatment is a small fraction of the harm it addresses.</t>
+    <t>Cost year 2017/18; unpublished Public Health England analysis for England (Black 2020, Part One evidence pack, p.14). Spend on treatment is a small fraction of the harm it addresses.</t>
   </si>
   <si>
     <t xml:space="preserve">H24</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">Domestic abuse</t>
   </si>
   <si>
-    <t xml:space="preserve">£66bn (≈£85bn in 2024 prices); £34,015 per victim</t>
+    <t>£66bn; £34,015 per victim</t>
   </si>
   <si>
     <t xml:space="preserve">Home Office cost-of-crime method</t>
@@ -1219,7 +1219,7 @@
     <t xml:space="preserve">Serious youth violence</t>
   </si>
   <si>
-    <t xml:space="preserve">About £1.3bn in 2018/19, up over 50% since 2014/15</t>
+    <t>About £1.3bn in 2018/19 (minimum £700m), up over 50% since 2014/15</t>
   </si>
   <si>
     <t xml:space="preserve">Academic estimate</t>
@@ -1228,13 +1228,13 @@
     <t xml:space="preserve">2018/19</t>
   </si>
   <si>
-    <t xml:space="preserve">Economics Observatory (2025), Youth violence in England and Wales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.economicsobservatory.com/youth-violence-in-england-and-wales-what-can-be-done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serious violence affecting children fell in 2024/25 on YEF's three core measures.</t>
+    <t>Youth Violence Commission (2020), Final report</t>
+  </si>
+  <si>
+    <t>https://wrap.warwick.ac.uk/id/eprint/154072/</t>
+  </si>
+  <si>
+    <t>In 2015/16 prices, using Home Office unit costs. £1.3bn adds violence not recorded by the police, estimated from the crime survey; £700m uses police-recorded crime only (pp.42, 52). Serious violence affecting children fell in 2024/25 on YEF's three core measures.</t>
   </si>
   <si>
     <t xml:space="preserve">I01</t>
@@ -2840,6 +2840,12 @@
   </si>
   <si>
     <t xml:space="preserve">Note: assumes burden falls in proportion to ACE prevalence, as Bellis et al. (2019) did for Europe and North America. DALYs and QALYs are different measures; the £70,000 conversion is a simplifying assumption.</t>
+  </si>
+  <si>
+    <t>Tax revenue only: £4.5bn from the 900,000 rise in sickness inactivity since 2020 (IPPR, using the OBR's £5,000 per person), plus the OBR's £3.0bn for in-work ill-health and £3.7bn for indirect effects on other taxes (p.28, note 9). Excludes the rise in benefit spending, which the OBR put at £6.8bn in 2023-24.</t>
+  </si>
+  <si>
+    <t>2015/16</t>
   </si>
 </sst>
 </file>
@@ -4683,7 +4689,7 @@
         <v>96</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="R19" s="10" t="s">
         <v>248</v>
@@ -4909,7 +4915,7 @@
         <v>81</v>
       </c>
       <c r="Q23" s="10" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="R23" s="10" t="s">
         <v>288</v>
@@ -4962,10 +4968,10 @@
         <v>295</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q24" s="10" t="s">
-        <v>296</v>
+        <v>202</v>
       </c>
       <c r="R24" s="10" t="s">
         <v>297</v>
@@ -5625,7 +5631,9 @@
       <c r="S36" s="11" t="s">
         <v>393</v>
       </c>
-      <c r="T36" s="10"/>
+      <c r="T36" s="10" t="s">
+        <v>938</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
@@ -5671,7 +5679,7 @@
         <v>70</v>
       </c>
       <c r="Q37" s="10" t="s">
-        <v>399</v>
+        <v>939</v>
       </c>
       <c r="R37" s="10" t="s">
         <v>400</v>
@@ -8737,7 +8745,7 @@
     <hyperlink ref="S34" r:id="rId33" display="https://www.nuffieldfjo.org.uk/resource/mothers-in-recurrent-care-proceedings-new-evidence-for-england-and-wales"/>
     <hyperlink ref="S35" r:id="rId34" display="https://cls.ucl.ac.uk/wp-content/uploads/2017/02/Children-of-care-leavers-policy-briefing.pdf"/>
     <hyperlink ref="S36" r:id="rId35" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
-    <hyperlink ref="S37" r:id="rId36" display="https://www.economicsobservatory.com/youth-violence-in-england-and-wales-what-can-be-done"/>
+    <hyperlink ref="S37" r:id="rId36" display="https://wrap.warwick.ac.uk/id/eprint/154072/"/>
     <hyperlink ref="S38" r:id="rId37" display="https://doi.org/10.1017/S0033291718001940"/>
     <hyperlink ref="S39" r:id="rId38" display="https://doi.org/10.1016/S2215-0366(25)00039-2"/>
     <hyperlink ref="S40" r:id="rId39" display="https://doi.org/10.1111/add.13160"/>

</xml_diff>

<commit_message>
Correct I31, H13 and I24 from their primary sources
Priority 2 checks of three grade D entries. I31 now cites Parsonage,
Grant and Stubbs (2016) and is regraded C; H13 is regraded C with Daley
et al.'s euro figures in the note; I24's note gives Park et al.'s 2009
price base. Approved by Stan Gilmour KPM FRSA on 27 September 2026.
Workbook cells updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="940">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="941">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -631,19 +631,19 @@
     <t xml:space="preserve">At least £17bn; about £17,000 more per adult per year</t>
   </si>
   <si>
-    <t xml:space="preserve">Secondary citation</t>
+    <t>Danish registry sibling comparison, scaled to the UK adult population</t>
   </si>
   <si>
     <t xml:space="preserve">not stated</t>
   </si>
   <si>
-    <t xml:space="preserve">NHS England, Independent ADHD Taskforce Part 1 (2025), citing Daley et al. (2019)</t>
+    <t>NHS England, Independent ADHD Taskforce Part 1 (2025), converting Daley et al. (2019)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.england.nhs.uk/long-read/report-of-the-independent-adhd-taskforce-part-1/</t>
   </si>
   <si>
-    <t xml:space="preserve">Per-adult figure derives from Danish sibling data. Taskforce links ADHD to early justice contact; 20–34% of NEET young people likely to have ADHD.</t>
+    <t>Daley et al. (2019) report in euros, from 2010 Danish register data: €20,135 more per adult with ADHD per year than a same-sex sibling (p.45), and €19,974m for the UK at 2.5% prevalence or €4,361m at 0.5% (Table 4, p.46), which the paper calls crude estimates. The Taskforce converted to pounds at an unstated rate and uses the higher prevalence. Taskforce links ADHD to early justice contact; 20–34% of NEET young people likely to have ADHD.</t>
   </si>
   <si>
     <t xml:space="preserve">H14</t>
@@ -1924,7 +1924,7 @@
     <t xml:space="preserve">https://doi.org/10.1111/eip.12149</t>
   </si>
   <si>
-    <t xml:space="preserve">Primary NICE page not seen.</t>
+    <t>Park et al. figures are in 2009 prices (p.145); the £2,087 is reduced lost productivity over years 1 to 3 (Table 3, p.147). The primary source for £15 per £1 is not traced: NHS England (2023) repeats it without a citation.</t>
   </si>
   <si>
     <t xml:space="preserve">I25</t>
@@ -2116,7 +2116,7 @@
     <t xml:space="preserve">Cost against saving</t>
   </si>
   <si>
-    <t xml:space="preserve">£2,700 per person; about £3,000 saved in mental health service use after one year</t>
+    <t>£2,700 per person (one-off); about £3,000 a year saved in mental health service use</t>
   </si>
   <si>
     <t xml:space="preserve">NHS, DWP</t>
@@ -2125,13 +2125,13 @@
     <t xml:space="preserve">NHS, DWP, the person</t>
   </si>
   <si>
-    <t xml:space="preserve">Secondary citation of Parsonage et al. (2016)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre for Mental Health (2022), Briefing 59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.centreformentalhealth.org.uk/wp-content/uploads/2022/09/CentreforMentalHealth_Briefing59_IPSforICSs.pdf</t>
+    <t>Charity economic analysis</t>
+  </si>
+  <si>
+    <t>Parsonage, Grant and Stubbs (2016), Priorities for mental health: economic report for the NHS England Mental Health Taskforce</t>
+  </si>
+  <si>
+    <t>https://www.centreformentalhealth.org.uk/wp-content/uploads/2018/09/priorities.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">I32</t>
@@ -2846,6 +2846,9 @@
   </si>
   <si>
     <t>2015/16</t>
+  </si>
+  <si>
+    <t>£3,000 a year is the lower end of the annualised savings (£3,000 to £4,000 a year) from three studies: £5,125 over 18 months, £20,000 over five years and £32,400 over ten years (p.34). Figures are in "today's prices", which the report does not define.</t>
   </si>
 </sst>
 </file>
@@ -4400,7 +4403,7 @@
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O14" s="10" t="s">
         <v>201</v>
@@ -7600,7 +7603,7 @@
         <v>698</v>
       </c>
       <c r="N68" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O68" s="10" t="s">
         <v>699</v>
@@ -7617,7 +7620,9 @@
       <c r="S68" s="11" t="s">
         <v>701</v>
       </c>
-      <c r="T68" s="10"/>
+      <c r="T68" s="10" t="s">
+        <v>940</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
@@ -8776,7 +8781,7 @@
     <hyperlink ref="S65" r:id="rId64" display="http://safelives.org.uk/research-policy-library/saving-lives-saving-money-report/"/>
     <hyperlink ref="S66" r:id="rId65" display="https://safelives.org.uk/about-domestic-abuse/responding-to-perpetrators/"/>
     <hyperlink ref="S67" r:id="rId66" display="https://assets.publishing.service.gov.uk/media/671a6fea603993b7a8f75db5/Housing_First_Cost_Benefit_Analysis_Report.pdf"/>
-    <hyperlink ref="S68" r:id="rId67" display="https://www.centreformentalhealth.org.uk/wp-content/uploads/2022/09/CentreforMentalHealth_Briefing59_IPSforICSs.pdf"/>
+    <hyperlink ref="S68" r:id="rId67" display="https://www.centreformentalhealth.org.uk/wp-content/uploads/2018/09/priorities.pdf"/>
     <hyperlink ref="S69" r:id="rId68" display="https://assets.publishing.service.gov.uk/media/5fa2d5e2d3bf7f03b3ee4925/Pause_-_Sussex.pdf"/>
     <hyperlink ref="S70" r:id="rId69" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10154457/"/>
     <hyperlink ref="S71" r:id="rId70" display="https://pubmed.ncbi.nlm.nih.gov/28356325/"/>

</xml_diff>

<commit_message>
Draft I36: Kurve kriegen (police-led early intervention, NRW)
New intervention entry from Prognos (2016), with the University of Kiel
impact evaluation (2015) in the note; grade C, result "Uncertain".
Rebasing exclusion added to rebase.json and a row inserted in the
workbook. Draft for Stan Gilmour KPM FRSA's approval; not for merge.
Also records the I31 page-number query.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$88</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$89</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1712" uniqueCount="941">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1732" uniqueCount="952">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -2849,6 +2849,39 @@
   </si>
   <si>
     <t>£3,000 a year is the lower end of the annualised savings (£3,000 to £4,000 a year) from three studies: £5,125 over 18 months, £20,000 over five years and £32,400 over ten years (p.34). Figures are in "today's prices", which the report does not define.</t>
+  </si>
+  <si>
+    <t>I36</t>
+  </si>
+  <si>
+    <t>Kurve kriegen (police-led early intervention, North Rhine-Westphalia)</t>
+  </si>
+  <si>
+    <t>Net benefit per €1 (modelled)</t>
+  </si>
+  <si>
+    <t>€3.23 net benefit per €1 (cautious scenario); €10.55 (optimistic scenario); about €13,354 per participant per year</t>
+  </si>
+  <si>
+    <t>NRW state (police)</t>
+  </si>
+  <si>
+    <t>Victims, justice system, youth welfare</t>
+  </si>
+  <si>
+    <t>Commissioned cost-benefit model using before-and-after data</t>
+  </si>
+  <si>
+    <t>Germany (North Rhine-Westphalia)</t>
+  </si>
+  <si>
+    <t>Prognos (2016), Cost-benefit analysis of the NRW crime-prevention initiative Kurve kriegen (management summary, in German)</t>
+  </si>
+  <si>
+    <t>https://www.kurvekriegen.nrw.de/sites/default/files/2021-11/2016_03_Prognos_KNA_Managementsummary.pdf</t>
+  </si>
+  <si>
+    <t>Prognos credits the programme with preventing 14 of 231 criminal careers (6%) in the cautious scenario and 40 (17%) in the optimistic one, valuing each at €1.66m to age 25 from a prototype offender it calls a realistic worst case; there is no comparison group (PDF pp.9, 10, 14–15). The gross return is €4.23 per €1. The University of Kiel's quasi-experimental impact evaluation (2015) found that participants' recorded offending stayed level while the comparison group's fell (p.204).</t>
   </si>
 </sst>
 </file>
@@ -3613,7 +3646,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T88"/>
+  <dimension ref="A1:T89"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -7868,61 +7901,69 @@
     </row>
     <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
-        <v>745</v>
+        <v>941</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>746</v>
+        <v>404</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E73" s="10"/>
+        <v>188</v>
+      </c>
+      <c r="E73" s="10" t="s">
+        <v>263</v>
+      </c>
       <c r="F73" s="10" t="s">
-        <v>747</v>
-      </c>
-      <c r="G73" s="10"/>
+        <v>217</v>
+      </c>
+      <c r="G73" s="10" t="s">
+        <v>134</v>
+      </c>
       <c r="H73" s="10" t="s">
-        <v>748</v>
+        <v>942</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>749</v>
+        <v>943</v>
       </c>
       <c r="J73" s="10" t="s">
-        <v>750</v>
-      </c>
-      <c r="K73" s="10"/>
-      <c r="L73" s="10"/>
-      <c r="M73" s="10"/>
+        <v>944</v>
+      </c>
+      <c r="K73" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="L73" s="10" t="s">
+        <v>945</v>
+      </c>
+      <c r="M73" s="10" t="s">
+        <v>946</v>
+      </c>
       <c r="N73" s="10" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>751</v>
+        <v>947</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>96</v>
+        <v>948</v>
       </c>
       <c r="Q73" s="10" t="s">
-        <v>296</v>
+        <v>202</v>
       </c>
       <c r="R73" s="10" t="s">
-        <v>752</v>
+        <v>949</v>
       </c>
       <c r="S73" s="11" t="s">
-        <v>753</v>
-      </c>
-      <c r="T73" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health.</t>
-        </is>
+        <v>950</v>
+      </c>
+      <c r="T73" s="10" t="s">
+        <v>951</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
-        <v>755</v>
+        <v>745</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>746</v>
@@ -7939,13 +7980,13 @@
       </c>
       <c r="G74" s="10"/>
       <c r="H74" s="10" t="s">
-        <v>756</v>
+        <v>748</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>757</v>
+        <v>749</v>
       </c>
       <c r="J74" s="10" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
       <c r="K74" s="10"/>
       <c r="L74" s="10"/>
@@ -7954,27 +7995,29 @@
         <v>10</v>
       </c>
       <c r="O74" s="10" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
       <c r="P74" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q74" s="10" t="s">
-        <v>139</v>
+        <v>296</v>
       </c>
       <c r="R74" s="10" t="s">
-        <v>760</v>
+        <v>752</v>
       </c>
       <c r="S74" s="11" t="s">
-        <v>761</v>
-      </c>
-      <c r="T74" s="10" t="s">
-        <v>762</v>
+        <v>753</v>
+      </c>
+      <c r="T74" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health.</t>
+        </is>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="s">
-        <v>763</v>
+        <v>755</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>746</v>
@@ -7991,13 +8034,13 @@
       </c>
       <c r="G75" s="10"/>
       <c r="H75" s="10" t="s">
-        <v>764</v>
+        <v>756</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="J75" s="10" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="K75" s="10"/>
       <c r="L75" s="10"/>
@@ -8006,25 +8049,27 @@
         <v>10</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q75" s="10" t="s">
-        <v>269</v>
+        <v>139</v>
       </c>
       <c r="R75" s="10" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="S75" s="11" t="s">
-        <v>768</v>
-      </c>
-      <c r="T75" s="10"/>
+        <v>761</v>
+      </c>
+      <c r="T75" s="10" t="s">
+        <v>762</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>746</v>
@@ -8041,13 +8086,13 @@
       </c>
       <c r="G76" s="10"/>
       <c r="H76" s="10" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>771</v>
+        <v>749</v>
       </c>
       <c r="J76" s="10" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="K76" s="10"/>
       <c r="L76" s="10"/>
@@ -8056,27 +8101,25 @@
         <v>10</v>
       </c>
       <c r="O76" s="10" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="P76" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q76" s="10" t="s">
         <v>269</v>
       </c>
       <c r="R76" s="10" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="S76" s="11" t="s">
-        <v>775</v>
-      </c>
-      <c r="T76" s="10" t="s">
-        <v>776</v>
-      </c>
+        <v>768</v>
+      </c>
+      <c r="T76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>746</v>
@@ -8093,42 +8136,42 @@
       </c>
       <c r="G77" s="10"/>
       <c r="H77" s="10" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
       <c r="I77" s="10" t="s">
         <v>771</v>
       </c>
       <c r="J77" s="10" t="s">
-        <v>779</v>
+        <v>772</v>
       </c>
       <c r="K77" s="10"/>
       <c r="L77" s="10"/>
       <c r="M77" s="10"/>
       <c r="N77" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>780</v>
+        <v>773</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q77" s="10" t="s">
-        <v>781</v>
+        <v>269</v>
       </c>
       <c r="R77" s="10" t="s">
-        <v>782</v>
+        <v>774</v>
       </c>
       <c r="S77" s="11" t="s">
-        <v>783</v>
+        <v>775</v>
       </c>
       <c r="T77" s="10" t="s">
-        <v>784</v>
+        <v>776</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10" t="s">
-        <v>785</v>
+        <v>777</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>746</v>
@@ -8145,13 +8188,13 @@
       </c>
       <c r="G78" s="10"/>
       <c r="H78" s="10" t="s">
-        <v>786</v>
+        <v>778</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>787</v>
+        <v>771</v>
       </c>
       <c r="J78" s="10" t="s">
-        <v>788</v>
+        <v>779</v>
       </c>
       <c r="K78" s="10"/>
       <c r="L78" s="10"/>
@@ -8160,27 +8203,27 @@
         <v>12</v>
       </c>
       <c r="O78" s="10" t="s">
-        <v>789</v>
+        <v>780</v>
       </c>
       <c r="P78" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q78" s="10" t="s">
-        <v>790</v>
+        <v>781</v>
       </c>
       <c r="R78" s="10" t="s">
-        <v>791</v>
+        <v>782</v>
       </c>
       <c r="S78" s="11" t="s">
-        <v>792</v>
+        <v>783</v>
       </c>
       <c r="T78" s="10" t="s">
-        <v>793</v>
+        <v>784</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
-        <v>794</v>
+        <v>785</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>746</v>
@@ -8197,96 +8240,94 @@
       </c>
       <c r="G79" s="10"/>
       <c r="H79" s="10" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>796</v>
+        <v>787</v>
       </c>
       <c r="J79" s="10" t="s">
-        <v>797</v>
+        <v>788</v>
       </c>
       <c r="K79" s="10"/>
       <c r="L79" s="10"/>
       <c r="M79" s="10"/>
       <c r="N79" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>798</v>
+        <v>789</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q79" s="10" t="s">
-        <v>658</v>
+        <v>790</v>
       </c>
       <c r="R79" s="10" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="S79" s="11" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
       <c r="T79" s="10" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>803</v>
+        <v>746</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E80" s="10"/>
       <c r="F80" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G80" s="10" t="s">
-        <v>91</v>
-      </c>
+        <v>747</v>
+      </c>
+      <c r="G80" s="10"/>
       <c r="H80" s="10" t="s">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>805</v>
+        <v>796</v>
       </c>
       <c r="J80" s="10" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="K80" s="10"/>
       <c r="L80" s="10"/>
       <c r="M80" s="10"/>
       <c r="N80" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O80" s="10" t="s">
-        <v>807</v>
+        <v>798</v>
       </c>
       <c r="P80" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q80" s="10" t="s">
-        <v>312</v>
+        <v>658</v>
       </c>
       <c r="R80" s="10" t="s">
-        <v>808</v>
-      </c>
-      <c r="S80" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
-        </is>
-      </c>
-      <c r="T80" s="10"/>
+        <v>799</v>
+      </c>
+      <c r="S80" s="11" t="s">
+        <v>800</v>
+      </c>
+      <c r="T80" s="10" t="s">
+        <v>801</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="s">
-        <v>810</v>
+        <v>802</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>803</v>
@@ -8299,19 +8340,19 @@
       </c>
       <c r="E81" s="10"/>
       <c r="F81" s="10" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="I81" s="10" t="s">
         <v>805</v>
       </c>
       <c r="J81" s="10" t="s">
-        <v>812</v>
+        <v>806</v>
       </c>
       <c r="K81" s="10"/>
       <c r="L81" s="10"/>
@@ -8329,95 +8370,97 @@
         <v>312</v>
       </c>
       <c r="R81" s="10" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="S81" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
         </is>
       </c>
       <c r="T81" s="10"/>
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E82" s="10"/>
       <c r="F82" s="10" t="s">
-        <v>90</v>
+        <v>176</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H82" s="10" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>817</v>
+        <v>805</v>
       </c>
       <c r="J82" s="10" t="s">
-        <v>818</v>
+        <v>812</v>
       </c>
       <c r="K82" s="10"/>
       <c r="L82" s="10"/>
       <c r="M82" s="10"/>
       <c r="N82" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O82" s="10" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
       <c r="P82" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q82" s="10" t="s">
-        <v>269</v>
+        <v>312</v>
       </c>
       <c r="R82" s="10" t="s">
-        <v>820</v>
-      </c>
-      <c r="S82" s="11" t="s">
-        <v>821</v>
+        <v>813</v>
+      </c>
+      <c r="S82" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+        </is>
       </c>
       <c r="T82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="s">
-        <v>822</v>
+        <v>815</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E83" s="10"/>
       <c r="F83" s="10" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>823</v>
+        <v>816</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>824</v>
+        <v>817</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>825</v>
+        <v>818</v>
       </c>
       <c r="K83" s="10"/>
       <c r="L83" s="10"/>
@@ -8426,241 +8469,241 @@
         <v>10</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>826</v>
+        <v>819</v>
       </c>
       <c r="P83" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q83" s="10" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="R83" s="10" t="s">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="S83" s="11" t="s">
-        <v>828</v>
-      </c>
-      <c r="T83" s="10" t="s">
-        <v>829</v>
-      </c>
+        <v>821</v>
+      </c>
+      <c r="T83" s="10"/>
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10" t="s">
-        <v>830</v>
+        <v>822</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>163</v>
+        <v>233</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="E84" s="10" t="s">
-        <v>111</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="E84" s="10"/>
       <c r="F84" s="10" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H84" s="10" t="s">
-        <v>831</v>
+        <v>823</v>
       </c>
       <c r="I84" s="10" t="s">
-        <v>832</v>
+        <v>824</v>
       </c>
       <c r="J84" s="10" t="s">
-        <v>833</v>
+        <v>825</v>
       </c>
       <c r="K84" s="10"/>
       <c r="L84" s="10"/>
       <c r="M84" s="10"/>
       <c r="N84" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O84" s="10" t="s">
-        <v>834</v>
+        <v>826</v>
       </c>
       <c r="P84" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q84" s="10" t="s">
         <v>247</v>
       </c>
       <c r="R84" s="10" t="s">
-        <v>835</v>
+        <v>827</v>
       </c>
       <c r="S84" s="11" t="s">
-        <v>836</v>
+        <v>828</v>
       </c>
       <c r="T84" s="10" t="s">
-        <v>837</v>
+        <v>829</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10" t="s">
-        <v>838</v>
+        <v>830</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>233</v>
+        <v>163</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="E85" s="10"/>
+        <v>164</v>
+      </c>
+      <c r="E85" s="10" t="s">
+        <v>111</v>
+      </c>
       <c r="F85" s="10" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>388</v>
+        <v>831</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
       <c r="J85" s="10" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
       <c r="K85" s="10"/>
       <c r="L85" s="10"/>
       <c r="M85" s="10"/>
       <c r="N85" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q85" s="10" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="R85" s="10" t="s">
-        <v>842</v>
+        <v>835</v>
       </c>
       <c r="S85" s="11" t="s">
-        <v>393</v>
-      </c>
-      <c r="T85" s="10"/>
+        <v>836</v>
+      </c>
+      <c r="T85" s="10" t="s">
+        <v>837</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>188</v>
+        <v>234</v>
       </c>
       <c r="E86" s="10"/>
       <c r="F86" s="10" t="s">
-        <v>76</v>
+        <v>176</v>
       </c>
       <c r="G86" s="10" t="s">
         <v>65</v>
       </c>
       <c r="H86" s="10" t="s">
-        <v>844</v>
+        <v>388</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>845</v>
+        <v>839</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>846</v>
+        <v>840</v>
       </c>
       <c r="K86" s="10"/>
       <c r="L86" s="10"/>
       <c r="M86" s="10"/>
       <c r="N86" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O86" s="10" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="P86" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q86" s="10" t="s">
-        <v>848</v>
+        <v>193</v>
       </c>
       <c r="R86" s="10" t="s">
-        <v>849</v>
+        <v>842</v>
       </c>
       <c r="S86" s="11" t="s">
-        <v>850</v>
-      </c>
-      <c r="T86" s="10" t="s">
-        <v>851</v>
-      </c>
+        <v>393</v>
+      </c>
+      <c r="T86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
-        <v>852</v>
+        <v>843</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>63</v>
+        <v>188</v>
       </c>
       <c r="E87" s="10"/>
       <c r="F87" s="10" t="s">
-        <v>176</v>
+        <v>76</v>
       </c>
       <c r="G87" s="10" t="s">
         <v>65</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>853</v>
+        <v>844</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="K87" s="10"/>
       <c r="L87" s="10"/>
       <c r="M87" s="10"/>
       <c r="N87" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>95</v>
+        <v>847</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q87" s="10" t="s">
-        <v>312</v>
+        <v>848</v>
       </c>
       <c r="R87" s="10" t="s">
-        <v>855</v>
+        <v>849</v>
       </c>
       <c r="S87" s="11" t="s">
-        <v>856</v>
-      </c>
-      <c r="T87" s="10"/>
+        <v>850</v>
+      </c>
+      <c r="T87" s="10" t="s">
+        <v>851</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="10" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>803</v>
@@ -8673,19 +8716,19 @@
       </c>
       <c r="E88" s="10"/>
       <c r="F88" s="10" t="s">
-        <v>64</v>
+        <v>176</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="H88" s="10" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="I88" s="10" t="s">
-        <v>859</v>
+        <v>839</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>860</v>
+        <v>854</v>
       </c>
       <c r="K88" s="10"/>
       <c r="L88" s="10"/>
@@ -8694,26 +8737,78 @@
         <v>14</v>
       </c>
       <c r="O88" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="P88" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q88" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="R88" s="10" t="s">
+        <v>855</v>
+      </c>
+      <c r="S88" s="11" t="s">
+        <v>856</v>
+      </c>
+      <c r="T88" s="10"/>
+    </row>
+    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="10" t="s">
+        <v>857</v>
+      </c>
+      <c r="B89" s="10" t="s">
+        <v>803</v>
+      </c>
+      <c r="C89" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D89" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E89" s="10"/>
+      <c r="F89" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G89" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H89" s="10" t="s">
+        <v>858</v>
+      </c>
+      <c r="I89" s="10" t="s">
+        <v>859</v>
+      </c>
+      <c r="J89" s="10" t="s">
+        <v>860</v>
+      </c>
+      <c r="K89" s="10"/>
+      <c r="L89" s="10"/>
+      <c r="M89" s="10"/>
+      <c r="N89" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="O89" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="P88" s="10" t="s">
+      <c r="P89" s="10" t="s">
         <v>861</v>
       </c>
-      <c r="Q88" s="10" t="s">
+      <c r="Q89" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="R88" s="10" t="s">
+      <c r="R89" s="10" t="s">
         <v>862</v>
       </c>
-      <c r="S88" s="11" t="s">
+      <c r="S89" s="11" t="s">
         <v>863</v>
       </c>
-      <c r="T88" s="10" t="s">
+      <c r="T89" s="10" t="s">
         <v>864</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T88"/>
+  <autoFilter ref="A1:T89"/>
   <hyperlinks>
     <hyperlink ref="S2" r:id="rId1" display="https://foundations.org.uk/our-work/publications/the-cost-of-late-intervention-eif-analysis-2016/"/>
     <hyperlink ref="S3" r:id="rId2" display="https://learning.nspcc.org.uk/research-resources/childrens-services-spending-reports"/>
@@ -8786,22 +8881,23 @@
     <hyperlink ref="S70" r:id="rId69" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10154457/"/>
     <hyperlink ref="S71" r:id="rId70" display="https://pubmed.ncbi.nlm.nih.gov/28356325/"/>
     <hyperlink ref="S72" r:id="rId71" display="https://www.health.org.uk/reports-and-analysis/analysis/investing-in-the-public-health-grant"/>
-    <hyperlink ref="S73" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
-    <hyperlink ref="S74" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
-    <hyperlink ref="S75" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
-    <hyperlink ref="S76" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
-    <hyperlink ref="S77" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
-    <hyperlink ref="S78" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
-    <hyperlink ref="S79" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
-    <hyperlink ref="S80" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
-    <hyperlink ref="S81" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
-    <hyperlink ref="S82" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
-    <hyperlink ref="S83" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
-    <hyperlink ref="S84" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
-    <hyperlink ref="S85" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
-    <hyperlink ref="S86" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
-    <hyperlink ref="S87" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
-    <hyperlink ref="S88" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
+    <hyperlink ref="S73" r:id="rId89" display="https://www.kurvekriegen.nrw.de/sites/default/files/2021-11/2016_03_Prognos_KNA_Managementsummary.pdf"/>
+    <hyperlink ref="S74" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
+    <hyperlink ref="S75" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
+    <hyperlink ref="S76" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
+    <hyperlink ref="S77" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
+    <hyperlink ref="S78" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
+    <hyperlink ref="S79" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
+    <hyperlink ref="S80" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
+    <hyperlink ref="S81" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
+    <hyperlink ref="S82" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
+    <hyperlink ref="S83" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
+    <hyperlink ref="S84" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
+    <hyperlink ref="S85" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
+    <hyperlink ref="S86" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
+    <hyperlink ref="S87" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
+    <hyperlink ref="S88" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
+    <hyperlink ref="S89" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Approve I36; add Kurve kriegen gap; correct I31 page reference
I36 and its rebasing exclusion approved by Stan Gilmour KPM FRSA on
27 September 2026. New known gap on police-identified early
intervention with no comparison-group economic evaluation, in
ledger.json and on the workbook's Read me sheet. I31 note now cites
p.35, matching the copy of the report at the I31 link, with the page
numbers in DATA-QUERIES.md corrected to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1732" uniqueCount="952">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="953">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -2848,7 +2848,7 @@
     <t>2015/16</t>
   </si>
   <si>
-    <t>£3,000 a year is the lower end of the annualised savings (£3,000 to £4,000 a year) from three studies: £5,125 over 18 months, £20,000 over five years and £32,400 over ten years (p.34). Figures are in "today's prices", which the report does not define.</t>
+    <t>£3,000 a year is the lower end of the annualised savings (£3,000 to £4,000 a year) from three studies: £5,125 over 18 months, £20,000 over five years and £32,400 over ten years (p.35). Figures are in "today's prices", which the report does not define.</t>
   </si>
   <si>
     <t>I36</t>
@@ -2882,6 +2882,9 @@
   </si>
   <si>
     <t>Prognos credits the programme with preventing 14 of 231 criminal careers (6%) in the cautious scenario and 40 (17%) in the optimistic one, valuing each at €1.66m to age 25 from a prototype offender it calls a realistic worst case; there is no comparison group (PDF pp.9, 10, 14–15). The gross return is €4.23 per €1. The University of Kiel's quasi-experimental impact evaluation (2015) found that participants' recorded offending stayed level while the comparison group's fell (p.204).</t>
+  </si>
+  <si>
+    <t>No economic evaluation with a comparison group of police-identified early intervention for children on the Kurve kriegen model; the German return is modelled from before-and-after data.</t>
   </si>
 </sst>
 </file>
@@ -3434,7 +3437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3628,6 +3631,12 @@
       <c r="A34" s="4"/>
       <c r="B34" s="5" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4"/>
+      <c r="B35" s="5" t="s">
+        <v>952</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trace I24's £15 per £1 to Knapp et al. (2014); correct P01 paragraph
I24 now cites Investing in recovery (Rethink Mental Illness, 2014),
p.10, as the source of "at least £15 per £1", regraded D to C. P01's
Green Book paragraph corrected to A1.64, with a note on where the 2026
edition's health guidance link leads. Workbook updated to match,
including the Parameters sheet. Approved by Stan Gilmour KPM FRSA on
27 September 2026. Closes the last open data query.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="953">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="954">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -1906,7 +1906,7 @@
     <t xml:space="preserve">Early intervention in psychosis</t>
   </si>
   <si>
-    <t xml:space="preserve">£15 per £1 over 10 years (secondary); £2,087 per person in employment and education gains over 3 years</t>
+    <t>At least £15 per £1 over 10 years; £2,087 per person in employment and education gains over 3 years</t>
   </si>
   <si>
     <t xml:space="preserve">NHS mental health</t>
@@ -1915,16 +1915,16 @@
     <t xml:space="preserve">NHS, DWP, economy</t>
   </si>
   <si>
-    <t xml:space="preserve">Secondary citation of NICE; Park et al. (2016) model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rethink Mental Illness briefing; Park, McCrone and Knapp (2016)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://doi.org/10.1111/eip.12149</t>
-  </si>
-  <si>
-    <t>Park et al. figures are in 2009 prices (p.145); the £2,087 is reduced lost productivity over years 1 to 3 (Table 3, p.147). The primary source for £15 per £1 is not traced: NHS England (2023) repeats it without a citation.</t>
+    <t>Charity-published model (Knapp et al. 2014); Park et al. (2016) model</t>
+  </si>
+  <si>
+    <t>Knapp et al. (2014), Investing in recovery (Rethink Mental Illness), p.10; Park, McCrone and Knapp (2016)</t>
+  </si>
+  <si>
+    <t>https://eprints.lse.ac.uk/56773/</t>
+  </si>
+  <si>
+    <t>Knapp et al. (2014) give net savings per person in 2012/13 prices (Table 2, p.10): £5,738 in year 1, £2,234 over years 1 to 3 and £6,780 over years 4 to 10. The calculation of the £15 per £1 ratio is not shown. NHS England (2023) and Rethink repeat the figure without a citation. Park et al. figures are in 2009 prices (p.145); the £2,087 is reduced lost productivity over years 1 to 3 (Table 3, p.147).</t>
   </si>
   <si>
     <t xml:space="preserve">I25</t>
@@ -2284,7 +2284,7 @@
     <t xml:space="preserve">Green Book guidance</t>
   </si>
   <si>
-    <t xml:space="preserve">HM Treasury Green Book (2022), Annex 1, para A1.63 (hosted copy)</t>
+    <t>HM Treasury Green Book (2022), Annex 1, para A1.64 (hosted copy)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf</t>
@@ -2638,7 +2638,7 @@
     <t xml:space="preserve">£ (2020/21 prices)</t>
   </si>
   <si>
-    <t xml:space="preserve">HM Treasury Green Book 2022, Annex 1, A1.63</t>
+    <t xml:space="preserve">HM Treasury Green Book 2022, Annex 1, A1.64</t>
   </si>
   <si>
     <t xml:space="preserve">Value of a WELLBY (central)</t>
@@ -2885,6 +2885,9 @@
   </si>
   <si>
     <t>No economic evaluation with a comparison group of police-identified early intervention for children on the Kurve kriegen model; the German return is modelled from before-and-after data.</t>
+  </si>
+  <si>
+    <t>Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health. The 2026 edition (para 8.57, p.62) links to a 2013 GOV.UK page holding the Department of Health guide Policy appraisal and health, which gives no current QALY value, so £70,000 in 2020/21 prices remains the latest published value.</t>
   </si>
 </sst>
 </file>
@@ -7217,7 +7220,7 @@
         <v>628</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O61" s="10" t="s">
         <v>629</v>
@@ -8018,10 +8021,8 @@
       <c r="S74" s="11" t="s">
         <v>753</v>
       </c>
-      <c r="T74" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health.</t>
-        </is>
+      <c r="T74" s="10" t="s">
+        <v>953</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8878,7 +8879,7 @@
     <hyperlink ref="S58" r:id="rId57" display="https://doi.org/10.1056/NEJMoa1203241"/>
     <hyperlink ref="S59" r:id="rId58" display="https://committees.parliament.uk/writtenevidence/72380/html/"/>
     <hyperlink ref="S60" r:id="rId59" display="https://www.ukyouth.org/wp-content/uploads/2022/11/Economic-Value-of-Youth-Work-Full-Report.pdf"/>
-    <hyperlink ref="S61" r:id="rId60" display="https://doi.org/10.1111/eip.12149"/>
+    <hyperlink ref="S61" r:id="rId60" display="https://eprints.lse.ac.uk/56773/"/>
     <hyperlink ref="S62" r:id="rId61" display="https://doi.org/10.1192/bjp.bp.111.107888"/>
     <hyperlink ref="S63" r:id="rId62" display="https://www.rand.org/pubs/research_briefs/RBA1271-1.html"/>
     <hyperlink ref="S64" r:id="rId63" display="https://www.gov.uk/government/publications/alcohol-and-drug-prevention-treatment-and-recovery-why-invest/alcohol-and-drug-prevention-treatment-and-recovery-why-invest"/>

</xml_diff>

<commit_message>
Add I37 NELI and I38 Talk of the Town; add youth justice SLT gap
Speech and language evidence reviewed for the ledger. I37 (NELI,
Reception) from West et al. (2022) and Dimova et al. (2020): grade A,
"Effective, cost unclear". I38 (Talk of the Town) from Thurston, Roseth
and O'Hare (2016): grade A, "No effect in UK trial". Both excluded from
rebasing. New known gap on the youth justice SLT study. Rows and gap
added to the workbook. Approved by Stan Gilmour KPM FRSA on
27 September 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$89</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$91</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="954">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1771" uniqueCount="972">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -2888,6 +2888,60 @@
   </si>
   <si>
     <t>Used to value health in social cost-benefit analysis. Differs from NICE's threshold, which is an opportunity cost. The 2026 Green Book no longer states a QALY value; it refers to supplementary guidance on health. The 2026 edition (para 8.57, p.62) links to a 2013 GOV.UK page holding the Department of Health guide Policy appraisal and health, which gives no current QALY value, so £70,000 in 2020/21 prices remains the latest published value.</t>
+  </si>
+  <si>
+    <t>I37</t>
+  </si>
+  <si>
+    <t>Nuffield Early Language Intervention (NELI), Reception</t>
+  </si>
+  <si>
+    <t>Effect on teacher-rated behaviour; cost per pupil</t>
+  </si>
+  <si>
+    <t>Behavioural adjustment d = 0.23 (teacher-rated); language skills 0.26 (0.17, 0.35); £58 per pupil per year over 3 years</t>
+  </si>
+  <si>
+    <t>Cluster RCT (193 schools, 1,173 children)</t>
+  </si>
+  <si>
+    <t>West et al. (2022), Journal of School Psychology; Dimova et al. (2020), EEF evaluation report</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.jsp.2022.04.006</t>
+  </si>
+  <si>
+    <t>Class teachers rated behaviour before and immediately after the 20-week programme (West et al. 2022, pp.334, 340); the gain was not mediated by gains in language (pp.341–342). The £58 covers materials and training for a one-form-entry school (£43 for two-form entry) and excludes about 120 hours of teaching assistant time (Dimova et al. 2020, pp.61–62, 65). No economic evaluation found. The trial did not measure exclusions or harm to staff. Three authors of West et al. are directors of OxEd and Assessment, which sells the LanguageScreen tool used to select children (p.343).</t>
+  </si>
+  <si>
+    <t>I38</t>
+  </si>
+  <si>
+    <t>Talk of the Town (whole-school speech, language and communication support)</t>
+  </si>
+  <si>
+    <t>Effect on reading comprehension and oral language</t>
+  </si>
+  <si>
+    <t>Reading comprehension −0.03 (−0.46, 0.40), n=2,696; oral language 0.11 (−1.19, 1.41), n=292; £50.97 per pupil per year</t>
+  </si>
+  <si>
+    <t>Cluster RCT (64 primary schools)</t>
+  </si>
+  <si>
+    <t>England (three local authorities)</t>
+  </si>
+  <si>
+    <t>Thurston, Roseth and O'Hare (2016), EEF evaluation report</t>
+  </si>
+  <si>
+    <t>https://files.eric.ed.gov/fulltext/ED581531.pdf</t>
+  </si>
+  <si>
+    <t>Pupils in Years 2 and 5; a whole-school model delivered by The Communication Trust that includes a speech and language therapist working in school. Outcomes were reading comprehension and oral language; the cost is £13,244.46 per school per year spread across all pupils (executive summary).</t>
+  </si>
+  <si>
+    <t>The youth justice study of speech and language therapy reviewed for the ledger (Gregory and Bryan, 2011) measures language, not offending or costs.</t>
   </si>
 </sst>
 </file>
@@ -3440,7 +3494,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3640,6 +3694,12 @@
       <c r="A35" s="4"/>
       <c r="B35" s="5" t="s">
         <v>952</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4"/>
+      <c r="B36" s="5" t="s">
+        <v>971</v>
       </c>
     </row>
   </sheetData>
@@ -3658,7 +3718,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T89"/>
+  <dimension ref="A1:T91"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -7975,111 +8035,125 @@
     </row>
     <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
-        <v>745</v>
+        <v>954</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>746</v>
+        <v>404</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>62</v>
+        <v>132</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E74" s="10"/>
+        <v>133</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>122</v>
+      </c>
       <c r="F74" s="10" t="s">
-        <v>747</v>
-      </c>
-      <c r="G74" s="10"/>
+        <v>153</v>
+      </c>
+      <c r="G74" s="10" t="s">
+        <v>91</v>
+      </c>
       <c r="H74" s="10" t="s">
-        <v>748</v>
+        <v>955</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>749</v>
+        <v>956</v>
       </c>
       <c r="J74" s="10" t="s">
-        <v>750</v>
-      </c>
-      <c r="K74" s="10"/>
-      <c r="L74" s="10"/>
+        <v>957</v>
+      </c>
+      <c r="K74" s="10" t="s">
+        <v>528</v>
+      </c>
+      <c r="L74" s="10" t="s">
+        <v>503</v>
+      </c>
       <c r="M74" s="10"/>
       <c r="N74" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O74" s="10" t="s">
-        <v>751</v>
+        <v>958</v>
       </c>
       <c r="P74" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q74" s="10" t="s">
-        <v>296</v>
+        <v>202</v>
       </c>
       <c r="R74" s="10" t="s">
-        <v>752</v>
+        <v>959</v>
       </c>
       <c r="S74" s="11" t="s">
-        <v>753</v>
+        <v>960</v>
       </c>
       <c r="T74" s="10" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="s">
-        <v>755</v>
+        <v>962</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>746</v>
+        <v>404</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>62</v>
+        <v>163</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E75" s="10"/>
+        <v>164</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>165</v>
+      </c>
       <c r="F75" s="10" t="s">
-        <v>747</v>
-      </c>
-      <c r="G75" s="10"/>
+        <v>153</v>
+      </c>
+      <c r="G75" s="10" t="s">
+        <v>91</v>
+      </c>
       <c r="H75" s="10" t="s">
-        <v>756</v>
+        <v>963</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>757</v>
+        <v>964</v>
       </c>
       <c r="J75" s="10" t="s">
-        <v>758</v>
-      </c>
-      <c r="K75" s="10"/>
+        <v>965</v>
+      </c>
+      <c r="K75" s="10" t="s">
+        <v>451</v>
+      </c>
       <c r="L75" s="10"/>
       <c r="M75" s="10"/>
       <c r="N75" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>759</v>
+        <v>966</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>96</v>
+        <v>967</v>
       </c>
       <c r="Q75" s="10" t="s">
-        <v>139</v>
+        <v>202</v>
       </c>
       <c r="R75" s="10" t="s">
-        <v>760</v>
+        <v>968</v>
       </c>
       <c r="S75" s="11" t="s">
-        <v>761</v>
+        <v>969</v>
       </c>
       <c r="T75" s="10" t="s">
-        <v>762</v>
+        <v>970</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10" t="s">
-        <v>763</v>
+        <v>745</v>
       </c>
       <c r="B76" s="10" t="s">
         <v>746</v>
@@ -8096,13 +8170,13 @@
       </c>
       <c r="G76" s="10"/>
       <c r="H76" s="10" t="s">
-        <v>764</v>
+        <v>748</v>
       </c>
       <c r="I76" s="10" t="s">
         <v>749</v>
       </c>
       <c r="J76" s="10" t="s">
-        <v>765</v>
+        <v>750</v>
       </c>
       <c r="K76" s="10"/>
       <c r="L76" s="10"/>
@@ -8111,25 +8185,27 @@
         <v>10</v>
       </c>
       <c r="O76" s="10" t="s">
-        <v>766</v>
+        <v>751</v>
       </c>
       <c r="P76" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q76" s="10" t="s">
-        <v>269</v>
+        <v>296</v>
       </c>
       <c r="R76" s="10" t="s">
-        <v>767</v>
+        <v>752</v>
       </c>
       <c r="S76" s="11" t="s">
-        <v>768</v>
-      </c>
-      <c r="T76" s="10"/>
+        <v>753</v>
+      </c>
+      <c r="T76" s="10" t="s">
+        <v>953</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10" t="s">
-        <v>769</v>
+        <v>755</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>746</v>
@@ -8146,13 +8222,13 @@
       </c>
       <c r="G77" s="10"/>
       <c r="H77" s="10" t="s">
-        <v>770</v>
+        <v>756</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>771</v>
+        <v>757</v>
       </c>
       <c r="J77" s="10" t="s">
-        <v>772</v>
+        <v>758</v>
       </c>
       <c r="K77" s="10"/>
       <c r="L77" s="10"/>
@@ -8161,27 +8237,27 @@
         <v>10</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>773</v>
+        <v>759</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q77" s="10" t="s">
-        <v>269</v>
+        <v>139</v>
       </c>
       <c r="R77" s="10" t="s">
-        <v>774</v>
+        <v>760</v>
       </c>
       <c r="S77" s="11" t="s">
-        <v>775</v>
+        <v>761</v>
       </c>
       <c r="T77" s="10" t="s">
-        <v>776</v>
+        <v>762</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10" t="s">
-        <v>777</v>
+        <v>763</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>746</v>
@@ -8198,42 +8274,40 @@
       </c>
       <c r="G78" s="10"/>
       <c r="H78" s="10" t="s">
-        <v>778</v>
+        <v>764</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>771</v>
+        <v>749</v>
       </c>
       <c r="J78" s="10" t="s">
-        <v>779</v>
+        <v>765</v>
       </c>
       <c r="K78" s="10"/>
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
       <c r="N78" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O78" s="10" t="s">
-        <v>780</v>
+        <v>766</v>
       </c>
       <c r="P78" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q78" s="10" t="s">
-        <v>781</v>
+        <v>269</v>
       </c>
       <c r="R78" s="10" t="s">
-        <v>782</v>
+        <v>767</v>
       </c>
       <c r="S78" s="11" t="s">
-        <v>783</v>
-      </c>
-      <c r="T78" s="10" t="s">
-        <v>784</v>
-      </c>
+        <v>768</v>
+      </c>
+      <c r="T78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
-        <v>785</v>
+        <v>769</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>746</v>
@@ -8250,42 +8324,42 @@
       </c>
       <c r="G79" s="10"/>
       <c r="H79" s="10" t="s">
-        <v>786</v>
+        <v>770</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>787</v>
+        <v>771</v>
       </c>
       <c r="J79" s="10" t="s">
-        <v>788</v>
+        <v>772</v>
       </c>
       <c r="K79" s="10"/>
       <c r="L79" s="10"/>
       <c r="M79" s="10"/>
       <c r="N79" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>789</v>
+        <v>773</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q79" s="10" t="s">
-        <v>790</v>
+        <v>269</v>
       </c>
       <c r="R79" s="10" t="s">
-        <v>791</v>
+        <v>774</v>
       </c>
       <c r="S79" s="11" t="s">
-        <v>792</v>
+        <v>775</v>
       </c>
       <c r="T79" s="10" t="s">
-        <v>793</v>
+        <v>776</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
-        <v>794</v>
+        <v>777</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>746</v>
@@ -8302,67 +8376,65 @@
       </c>
       <c r="G80" s="10"/>
       <c r="H80" s="10" t="s">
-        <v>795</v>
+        <v>778</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>796</v>
+        <v>771</v>
       </c>
       <c r="J80" s="10" t="s">
-        <v>797</v>
+        <v>779</v>
       </c>
       <c r="K80" s="10"/>
       <c r="L80" s="10"/>
       <c r="M80" s="10"/>
       <c r="N80" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O80" s="10" t="s">
-        <v>798</v>
+        <v>780</v>
       </c>
       <c r="P80" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q80" s="10" t="s">
-        <v>658</v>
+        <v>781</v>
       </c>
       <c r="R80" s="10" t="s">
-        <v>799</v>
+        <v>782</v>
       </c>
       <c r="S80" s="11" t="s">
-        <v>800</v>
+        <v>783</v>
       </c>
       <c r="T80" s="10" t="s">
-        <v>801</v>
+        <v>784</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="s">
-        <v>802</v>
+        <v>785</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>803</v>
+        <v>746</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E81" s="10"/>
       <c r="F81" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G81" s="10" t="s">
-        <v>91</v>
-      </c>
+        <v>747</v>
+      </c>
+      <c r="G81" s="10"/>
       <c r="H81" s="10" t="s">
-        <v>804</v>
+        <v>786</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>805</v>
+        <v>787</v>
       </c>
       <c r="J81" s="10" t="s">
-        <v>806</v>
+        <v>788</v>
       </c>
       <c r="K81" s="10"/>
       <c r="L81" s="10"/>
@@ -8371,90 +8443,88 @@
         <v>12</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>807</v>
+        <v>789</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q81" s="10" t="s">
-        <v>312</v>
+        <v>790</v>
       </c>
       <c r="R81" s="10" t="s">
-        <v>808</v>
-      </c>
-      <c r="S81" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
-        </is>
-      </c>
-      <c r="T81" s="10"/>
+        <v>791</v>
+      </c>
+      <c r="S81" s="11" t="s">
+        <v>792</v>
+      </c>
+      <c r="T81" s="10" t="s">
+        <v>793</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10" t="s">
-        <v>810</v>
+        <v>794</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>803</v>
+        <v>746</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E82" s="10"/>
       <c r="F82" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="G82" s="10" t="s">
-        <v>65</v>
-      </c>
+        <v>747</v>
+      </c>
+      <c r="G82" s="10"/>
       <c r="H82" s="10" t="s">
-        <v>811</v>
+        <v>795</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>805</v>
+        <v>796</v>
       </c>
       <c r="J82" s="10" t="s">
-        <v>812</v>
+        <v>797</v>
       </c>
       <c r="K82" s="10"/>
       <c r="L82" s="10"/>
       <c r="M82" s="10"/>
       <c r="N82" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O82" s="10" t="s">
-        <v>807</v>
+        <v>798</v>
       </c>
       <c r="P82" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q82" s="10" t="s">
-        <v>312</v>
+        <v>658</v>
       </c>
       <c r="R82" s="10" t="s">
-        <v>813</v>
-      </c>
-      <c r="S82" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
-        </is>
-      </c>
-      <c r="T82" s="10"/>
+        <v>799</v>
+      </c>
+      <c r="S82" s="11" t="s">
+        <v>800</v>
+      </c>
+      <c r="T82" s="10" t="s">
+        <v>801</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="s">
-        <v>815</v>
+        <v>802</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E83" s="10"/>
       <c r="F83" s="10" t="s">
@@ -8464,40 +8534,42 @@
         <v>91</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>816</v>
+        <v>804</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>817</v>
+        <v>805</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>818</v>
+        <v>806</v>
       </c>
       <c r="K83" s="10"/>
       <c r="L83" s="10"/>
       <c r="M83" s="10"/>
       <c r="N83" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q83" s="10" t="s">
-        <v>269</v>
+        <v>312</v>
       </c>
       <c r="R83" s="10" t="s">
-        <v>820</v>
-      </c>
-      <c r="S83" s="11" t="s">
-        <v>821</v>
+        <v>808</v>
+      </c>
+      <c r="S83" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
+        </is>
       </c>
       <c r="T83" s="10"/>
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10" t="s">
-        <v>822</v>
+        <v>810</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>803</v>
@@ -8516,98 +8588,94 @@
         <v>65</v>
       </c>
       <c r="H84" s="10" t="s">
-        <v>823</v>
+        <v>811</v>
       </c>
       <c r="I84" s="10" t="s">
-        <v>824</v>
+        <v>805</v>
       </c>
       <c r="J84" s="10" t="s">
-        <v>825</v>
+        <v>812</v>
       </c>
       <c r="K84" s="10"/>
       <c r="L84" s="10"/>
       <c r="M84" s="10"/>
       <c r="N84" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O84" s="10" t="s">
-        <v>826</v>
+        <v>807</v>
       </c>
       <c r="P84" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q84" s="10" t="s">
-        <v>247</v>
+        <v>312</v>
       </c>
       <c r="R84" s="10" t="s">
-        <v>827</v>
-      </c>
-      <c r="S84" s="11" t="s">
-        <v>828</v>
-      </c>
-      <c r="T84" s="10" t="s">
-        <v>829</v>
-      </c>
+        <v>813</v>
+      </c>
+      <c r="S84" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+        </is>
+      </c>
+      <c r="T84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10" t="s">
-        <v>830</v>
+        <v>815</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>163</v>
+        <v>62</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>111</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="E85" s="10"/>
       <c r="F85" s="10" t="s">
-        <v>153</v>
+        <v>90</v>
       </c>
       <c r="G85" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>831</v>
+        <v>816</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>832</v>
+        <v>817</v>
       </c>
       <c r="J85" s="10" t="s">
-        <v>833</v>
+        <v>818</v>
       </c>
       <c r="K85" s="10"/>
       <c r="L85" s="10"/>
       <c r="M85" s="10"/>
       <c r="N85" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>834</v>
+        <v>819</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q85" s="10" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="R85" s="10" t="s">
-        <v>835</v>
+        <v>820</v>
       </c>
       <c r="S85" s="11" t="s">
-        <v>836</v>
-      </c>
-      <c r="T85" s="10" t="s">
-        <v>837</v>
-      </c>
+        <v>821</v>
+      </c>
+      <c r="T85" s="10"/>
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10" t="s">
-        <v>838</v>
+        <v>822</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>803</v>
@@ -8626,65 +8694,69 @@
         <v>65</v>
       </c>
       <c r="H86" s="10" t="s">
-        <v>388</v>
+        <v>823</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>839</v>
+        <v>824</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>840</v>
+        <v>825</v>
       </c>
       <c r="K86" s="10"/>
       <c r="L86" s="10"/>
       <c r="M86" s="10"/>
       <c r="N86" s="10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O86" s="10" t="s">
-        <v>841</v>
+        <v>826</v>
       </c>
       <c r="P86" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q86" s="10" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="R86" s="10" t="s">
-        <v>842</v>
+        <v>827</v>
       </c>
       <c r="S86" s="11" t="s">
-        <v>393</v>
-      </c>
-      <c r="T86" s="10"/>
+        <v>828</v>
+      </c>
+      <c r="T86" s="10" t="s">
+        <v>829</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
-        <v>843</v>
+        <v>830</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E87" s="10"/>
+        <v>164</v>
+      </c>
+      <c r="E87" s="10" t="s">
+        <v>111</v>
+      </c>
       <c r="F87" s="10" t="s">
-        <v>76</v>
+        <v>153</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>844</v>
+        <v>831</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>845</v>
+        <v>832</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>846</v>
+        <v>833</v>
       </c>
       <c r="K87" s="10"/>
       <c r="L87" s="10"/>
@@ -8693,36 +8765,36 @@
         <v>12</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>847</v>
+        <v>834</v>
       </c>
       <c r="P87" s="10" t="s">
         <v>81</v>
       </c>
       <c r="Q87" s="10" t="s">
-        <v>848</v>
+        <v>247</v>
       </c>
       <c r="R87" s="10" t="s">
-        <v>849</v>
+        <v>835</v>
       </c>
       <c r="S87" s="11" t="s">
-        <v>850</v>
+        <v>836</v>
       </c>
       <c r="T87" s="10" t="s">
-        <v>851</v>
+        <v>837</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="10" t="s">
-        <v>852</v>
+        <v>838</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E88" s="10"/>
       <c r="F88" s="10" t="s">
@@ -8732,13 +8804,13 @@
         <v>65</v>
       </c>
       <c r="H88" s="10" t="s">
-        <v>853</v>
+        <v>388</v>
       </c>
       <c r="I88" s="10" t="s">
         <v>839</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>854</v>
+        <v>840</v>
       </c>
       <c r="K88" s="10"/>
       <c r="L88" s="10"/>
@@ -8747,78 +8819,184 @@
         <v>14</v>
       </c>
       <c r="O88" s="10" t="s">
-        <v>95</v>
+        <v>841</v>
       </c>
       <c r="P88" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q88" s="10" t="s">
-        <v>312</v>
+        <v>193</v>
       </c>
       <c r="R88" s="10" t="s">
-        <v>855</v>
+        <v>842</v>
       </c>
       <c r="S88" s="11" t="s">
-        <v>856</v>
+        <v>393</v>
       </c>
       <c r="T88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="10" t="s">
-        <v>857</v>
+        <v>843</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>63</v>
+        <v>188</v>
       </c>
       <c r="E89" s="10"/>
       <c r="F89" s="10" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>858</v>
+        <v>844</v>
       </c>
       <c r="I89" s="10" t="s">
-        <v>859</v>
+        <v>845</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>860</v>
+        <v>846</v>
       </c>
       <c r="K89" s="10"/>
       <c r="L89" s="10"/>
       <c r="M89" s="10"/>
       <c r="N89" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="O89" s="10" t="s">
+        <v>847</v>
+      </c>
+      <c r="P89" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q89" s="10" t="s">
+        <v>848</v>
+      </c>
+      <c r="R89" s="10" t="s">
+        <v>849</v>
+      </c>
+      <c r="S89" s="11" t="s">
+        <v>850</v>
+      </c>
+      <c r="T89" s="10" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="10" t="s">
+        <v>852</v>
+      </c>
+      <c r="B90" s="10" t="s">
+        <v>803</v>
+      </c>
+      <c r="C90" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E90" s="10"/>
+      <c r="F90" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="G90" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H90" s="10" t="s">
+        <v>853</v>
+      </c>
+      <c r="I90" s="10" t="s">
+        <v>839</v>
+      </c>
+      <c r="J90" s="10" t="s">
+        <v>854</v>
+      </c>
+      <c r="K90" s="10"/>
+      <c r="L90" s="10"/>
+      <c r="M90" s="10"/>
+      <c r="N90" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="O89" s="10" t="s">
+      <c r="O90" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="P90" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q90" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="R90" s="10" t="s">
+        <v>855</v>
+      </c>
+      <c r="S90" s="11" t="s">
+        <v>856</v>
+      </c>
+      <c r="T90" s="10"/>
+    </row>
+    <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="10" t="s">
+        <v>857</v>
+      </c>
+      <c r="B91" s="10" t="s">
+        <v>803</v>
+      </c>
+      <c r="C91" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D91" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E91" s="10"/>
+      <c r="F91" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G91" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H91" s="10" t="s">
+        <v>858</v>
+      </c>
+      <c r="I91" s="10" t="s">
+        <v>859</v>
+      </c>
+      <c r="J91" s="10" t="s">
+        <v>860</v>
+      </c>
+      <c r="K91" s="10"/>
+      <c r="L91" s="10"/>
+      <c r="M91" s="10"/>
+      <c r="N91" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="O91" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="P89" s="10" t="s">
+      <c r="P91" s="10" t="s">
         <v>861</v>
       </c>
-      <c r="Q89" s="10" t="s">
+      <c r="Q91" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="R89" s="10" t="s">
+      <c r="R91" s="10" t="s">
         <v>862</v>
       </c>
-      <c r="S89" s="11" t="s">
+      <c r="S91" s="11" t="s">
         <v>863</v>
       </c>
-      <c r="T89" s="10" t="s">
+      <c r="T91" s="10" t="s">
         <v>864</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T89"/>
+  <autoFilter ref="A1:T91"/>
   <hyperlinks>
     <hyperlink ref="S2" r:id="rId1" display="https://foundations.org.uk/our-work/publications/the-cost-of-late-intervention-eif-analysis-2016/"/>
     <hyperlink ref="S3" r:id="rId2" display="https://learning.nspcc.org.uk/research-resources/childrens-services-spending-reports"/>
@@ -8892,22 +9070,24 @@
     <hyperlink ref="S71" r:id="rId70" display="https://pubmed.ncbi.nlm.nih.gov/28356325/"/>
     <hyperlink ref="S72" r:id="rId71" display="https://www.health.org.uk/reports-and-analysis/analysis/investing-in-the-public-health-grant"/>
     <hyperlink ref="S73" r:id="rId89" display="https://www.kurvekriegen.nrw.de/sites/default/files/2021-11/2016_03_Prognos_KNA_Managementsummary.pdf"/>
-    <hyperlink ref="S74" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
-    <hyperlink ref="S75" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
-    <hyperlink ref="S76" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
-    <hyperlink ref="S77" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
-    <hyperlink ref="S78" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
-    <hyperlink ref="S79" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
-    <hyperlink ref="S80" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
-    <hyperlink ref="S81" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
-    <hyperlink ref="S82" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
-    <hyperlink ref="S83" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
-    <hyperlink ref="S84" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
-    <hyperlink ref="S85" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
-    <hyperlink ref="S86" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
-    <hyperlink ref="S87" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
-    <hyperlink ref="S88" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
-    <hyperlink ref="S89" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
+    <hyperlink ref="S74" r:id="rId90" display="https://doi.org/10.1016/j.jsp.2022.04.006"/>
+    <hyperlink ref="S75" r:id="rId91" display="https://files.eric.ed.gov/fulltext/ED581531.pdf"/>
+    <hyperlink ref="S76" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
+    <hyperlink ref="S77" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
+    <hyperlink ref="S78" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
+    <hyperlink ref="S79" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
+    <hyperlink ref="S80" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
+    <hyperlink ref="S81" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
+    <hyperlink ref="S82" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
+    <hyperlink ref="S83" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
+    <hyperlink ref="S84" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
+    <hyperlink ref="S85" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
+    <hyperlink ref="S86" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
+    <hyperlink ref="S87" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
+    <hyperlink ref="S88" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
+    <hyperlink ref="S89" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
+    <hyperlink ref="S90" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
+    <hyperlink ref="S91" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add H37: language impairment among children in custody
Prevalence entry from Hughes et al. (2017), JCPP: 47% significantly
below average in an aspect of language and 28% impaired among 93 males
aged 15-18 in a young offender institution in England. Grade B;
excluded from rebasing (prevalence). Row added to the workbook.
Approved by Stan Gilmour KPM FRSA on 27 September 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/prevention-returns-ledger.xlsx
+++ b/public/downloads/prevention-returns-ledger.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$91</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Ledger!$A$1:$T$92</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1771" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1788" uniqueCount="978">
   <si>
     <t xml:space="preserve">Prevention Returns Ledger</t>
   </si>
@@ -2942,6 +2942,24 @@
   </si>
   <si>
     <t>The youth justice study of speech and language therapy reviewed for the ledger (Gregory and Bryan, 2011) measures language, not offending or costs.</t>
+  </si>
+  <si>
+    <t>H37</t>
+  </si>
+  <si>
+    <t>Language impairment among children in custody</t>
+  </si>
+  <si>
+    <t>47% significantly below average in an aspect of language; 28% impaired; 7 of 26 with an impairment had received speech and language therapy</t>
+  </si>
+  <si>
+    <t>Hughes et al. (2017), JCPP</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/jcpp.12791</t>
+  </si>
+  <si>
+    <t>Consecutive admissions to a young offender institution in North West England; 93 of 279 approached took part (pp.1107–1108). Of the 26 with an impairment, 76% had been excluded from school and 54% had attended a non-mainstream school (Table 5, p.1109). An earlier study of 58 young men aged 15–17 found 66–90% below average on language subtests (Bryan, Freer and Furlong 2007, p.505).</t>
   </si>
 </sst>
 </file>
@@ -3718,7 +3736,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T91"/>
+  <dimension ref="A1:T92"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5801,69 +5819,63 @@
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>403</v>
+        <v>972</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>404</v>
+        <v>61</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>87</v>
+        <v>187</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>88</v>
+        <v>188</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>90</v>
+        <v>217</v>
       </c>
       <c r="G38" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>405</v>
+        <v>973</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>406</v>
+        <v>113</v>
       </c>
       <c r="J38" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="K38" s="10" t="s">
-        <v>408</v>
-      </c>
-      <c r="L38" s="10" t="s">
-        <v>409</v>
-      </c>
-      <c r="M38" s="10" t="s">
-        <v>410</v>
-      </c>
+        <v>974</v>
+      </c>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
       <c r="N38" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O38" s="10" t="s">
-        <v>411</v>
+        <v>228</v>
       </c>
       <c r="P38" s="10" t="s">
-        <v>412</v>
+        <v>81</v>
       </c>
       <c r="Q38" s="10" t="s">
-        <v>202</v>
+        <v>117</v>
       </c>
       <c r="R38" s="10" t="s">
-        <v>413</v>
+        <v>975</v>
       </c>
       <c r="S38" s="11" t="s">
-        <v>414</v>
+        <v>976</v>
       </c>
       <c r="T38" s="10" t="s">
-        <v>415</v>
+        <v>977</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>416</v>
+        <v>403</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>404</v>
@@ -5884,114 +5896,114 @@
         <v>91</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>406</v>
       </c>
       <c r="J39" s="10" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="M39" s="10" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="N39" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O39" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="P39" s="10" t="s">
+        <v>412</v>
+      </c>
+      <c r="Q39" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="R39" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="S39" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="T39" s="10" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="J40" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="K40" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="L40" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="M40" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="N40" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="O40" s="10" t="s">
         <v>422</v>
       </c>
-      <c r="P39" s="10" t="s">
+      <c r="P40" s="10" t="s">
         <v>423</v>
       </c>
-      <c r="Q39" s="10" t="s">
+      <c r="Q40" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="R39" s="10" t="inlineStr">
+      <c r="R40" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Ullah et al. (2025), Lancet Psychiatry (ROSHNI-2 economic evaluation)</t>
         </is>
       </c>
-      <c r="S39" s="11" t="inlineStr">
+      <c r="S40" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">https://doi.org/10.1016/S2215-0366(25)00039-2</t>
         </is>
       </c>
-      <c r="T39" s="10" t="s">
+      <c r="T40" s="10" t="s">
         <v>426</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10" t="s">
-        <v>427</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="F40" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="H40" s="10" t="s">
-        <v>428</v>
-      </c>
-      <c r="I40" s="10" t="s">
-        <v>429</v>
-      </c>
-      <c r="J40" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="K40" s="10" t="s">
-        <v>419</v>
-      </c>
-      <c r="L40" s="10" t="s">
-        <v>431</v>
-      </c>
-      <c r="M40" s="10" t="s">
-        <v>421</v>
-      </c>
-      <c r="N40" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="O40" s="10" t="s">
-        <v>432</v>
-      </c>
-      <c r="P40" s="10" t="s">
-        <v>433</v>
-      </c>
-      <c r="Q40" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="R40" s="10" t="s">
-        <v>434</v>
-      </c>
-      <c r="S40" s="11" t="s">
-        <v>435</v>
-      </c>
-      <c r="T40" s="10" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>404</v>
@@ -6012,60 +6024,60 @@
         <v>91</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>406</v>
+        <v>429</v>
       </c>
       <c r="J41" s="10" t="s">
-        <v>439</v>
+        <v>430</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="L41" s="10" t="s">
         <v>431</v>
       </c>
       <c r="M41" s="10" t="s">
-        <v>440</v>
+        <v>421</v>
       </c>
       <c r="N41" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>441</v>
+        <v>432</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="Q41" s="10" t="s">
-        <v>443</v>
+        <v>202</v>
       </c>
       <c r="R41" s="10" t="s">
-        <v>444</v>
+        <v>434</v>
       </c>
       <c r="S41" s="11" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="T41" s="10" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>132</v>
+        <v>87</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>133</v>
+        <v>88</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="F42" s="10" t="s">
         <v>90</v>
@@ -6074,110 +6086,110 @@
         <v>91</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>449</v>
+        <v>406</v>
       </c>
       <c r="J42" s="10" t="s">
-        <v>450</v>
+        <v>439</v>
       </c>
       <c r="K42" s="10" t="s">
-        <v>451</v>
+        <v>408</v>
       </c>
       <c r="L42" s="10" t="s">
-        <v>452</v>
-      </c>
-      <c r="M42" s="10"/>
+        <v>431</v>
+      </c>
+      <c r="M42" s="10" t="s">
+        <v>440</v>
+      </c>
       <c r="N42" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O42" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="P42" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="Q42" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="R42" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="S42" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="T42" s="10" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>447</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>448</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="J43" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="K43" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="L43" s="10" t="s">
+        <v>452</v>
+      </c>
+      <c r="M43" s="10"/>
+      <c r="N43" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="O43" s="10" t="s">
         <v>453</v>
       </c>
-      <c r="P42" s="10" t="s">
+      <c r="P43" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="Q42" s="10" t="inlineStr">
+      <c r="Q43" s="10" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="R42" s="10" t="s">
+      <c r="R43" s="10" t="s">
         <v>455</v>
       </c>
-      <c r="S42" s="11" t="s">
+      <c r="S43" s="11" t="s">
         <v>456</v>
       </c>
-      <c r="T42" s="10" t="s">
+      <c r="T43" s="10" t="s">
         <v>457</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="s">
-        <v>458</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="F43" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>459</v>
-      </c>
-      <c r="I43" s="10" t="s">
-        <v>460</v>
-      </c>
-      <c r="J43" s="10" t="s">
-        <v>461</v>
-      </c>
-      <c r="K43" s="10" t="s">
-        <v>419</v>
-      </c>
-      <c r="L43" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="M43" s="10" t="s">
-        <v>463</v>
-      </c>
-      <c r="N43" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="O43" s="10" t="s">
-        <v>464</v>
-      </c>
-      <c r="P43" s="10" t="s">
-        <v>465</v>
-      </c>
-      <c r="Q43" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="R43" s="10" t="s">
-        <v>466</v>
-      </c>
-      <c r="S43" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="T43" s="10" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>404</v>
@@ -6192,118 +6204,118 @@
         <v>165</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="G44" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H44" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="I44" s="10" t="s">
+        <v>460</v>
+      </c>
+      <c r="J44" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="K44" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="L44" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="M44" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="N44" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="O44" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="P44" s="10" t="s">
+        <v>465</v>
+      </c>
+      <c r="Q44" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="R44" s="10" t="s">
+        <v>466</v>
+      </c>
+      <c r="S44" s="11" t="s">
+        <v>467</v>
+      </c>
+      <c r="T44" s="10" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>470</v>
       </c>
-      <c r="I44" s="10" t="s">
+      <c r="I45" s="10" t="s">
         <v>471</v>
       </c>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="J45" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">£1,177 per participant; public-sector savings 2.8–6.1 times cost; societal savings £16,435 over 25 years; payback 5–8 years</t>
         </is>
       </c>
-      <c r="K44" s="10" t="s">
-        <v>473</v>
-      </c>
-      <c r="L44" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="M44" s="10" t="s">
-        <v>474</v>
-      </c>
-      <c r="N44" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="O44" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="P44" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q44" s="10" t="s">
-        <v>475</v>
-      </c>
-      <c r="R44" s="10" t="s">
-        <v>476</v>
-      </c>
-      <c r="S44" s="11" t="s">
-        <v>477</v>
-      </c>
-      <c r="T44" s="10" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="10" t="s">
-        <v>479</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="C45" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="E45" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="F45" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G45" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="I45" s="10" t="s">
-        <v>481</v>
-      </c>
-      <c r="J45" s="10" t="s">
-        <v>482</v>
-      </c>
       <c r="K45" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>483</v>
+        <v>462</v>
       </c>
       <c r="M45" s="10" t="s">
-        <v>484</v>
+        <v>474</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>485</v>
+        <v>126</v>
       </c>
       <c r="P45" s="10" t="s">
         <v>81</v>
       </c>
       <c r="Q45" s="10" t="s">
-        <v>256</v>
+        <v>475</v>
       </c>
       <c r="R45" s="10" t="s">
-        <v>486</v>
+        <v>476</v>
       </c>
       <c r="S45" s="11" t="s">
-        <v>487</v>
+        <v>477</v>
       </c>
       <c r="T45" s="10" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>489</v>
+        <v>479</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>404</v>
@@ -6315,117 +6327,117 @@
         <v>133</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>490</v>
+        <v>480</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>491</v>
+        <v>481</v>
       </c>
       <c r="J46" s="10" t="s">
-        <v>492</v>
+        <v>482</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>493</v>
+        <v>473</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="M46" s="10"/>
+        <v>483</v>
+      </c>
+      <c r="M46" s="10" t="s">
+        <v>484</v>
+      </c>
       <c r="N46" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O46" s="10" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
       <c r="P46" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q46" s="10" t="s">
-        <v>495</v>
+        <v>256</v>
       </c>
       <c r="R46" s="10" t="s">
-        <v>496</v>
+        <v>486</v>
       </c>
       <c r="S46" s="11" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="T46" s="10" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>499</v>
+        <v>489</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>165</v>
+        <v>111</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>153</v>
+        <v>90</v>
       </c>
       <c r="G47" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
       <c r="J47" s="10" t="s">
-        <v>502</v>
+        <v>492</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="L47" s="10" t="s">
-        <v>503</v>
-      </c>
-      <c r="M47" s="10" t="s">
-        <v>504</v>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="M47" s="10"/>
       <c r="N47" s="10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>126</v>
+        <v>494</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q47" s="10" t="s">
-        <v>106</v>
+        <v>495</v>
       </c>
       <c r="R47" s="10" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
       <c r="S47" s="11" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="T47" s="10" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10" t="s">
-        <v>508</v>
+        <v>499</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>404</v>
@@ -6443,16 +6455,16 @@
         <v>153</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>134</v>
+        <v>91</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>501</v>
       </c>
       <c r="J48" s="10" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="K48" s="10" t="s">
         <v>473</v>
@@ -6461,7 +6473,7 @@
         <v>503</v>
       </c>
       <c r="M48" s="10" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="N48" s="10" t="s">
         <v>14</v>
@@ -6470,7 +6482,7 @@
         <v>126</v>
       </c>
       <c r="P48" s="10" t="s">
-        <v>512</v>
+        <v>81</v>
       </c>
       <c r="Q48" s="10" t="s">
         <v>106</v>
@@ -6482,12 +6494,12 @@
         <v>506</v>
       </c>
       <c r="T48" s="10" t="s">
-        <v>513</v>
+        <v>507</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>404</v>
@@ -6502,66 +6514,66 @@
         <v>165</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>395</v>
+        <v>153</v>
       </c>
       <c r="G49" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>516</v>
+        <v>501</v>
       </c>
       <c r="J49" s="10" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="K49" s="10" t="s">
-        <v>518</v>
+        <v>473</v>
       </c>
       <c r="L49" s="10" t="s">
         <v>503</v>
       </c>
       <c r="M49" s="10" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>520</v>
+        <v>126</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="Q49" s="10" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="R49" s="10" t="s">
-        <v>522</v>
+        <v>505</v>
       </c>
       <c r="S49" s="11" t="s">
-        <v>523</v>
+        <v>506</v>
       </c>
       <c r="T49" s="10" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
-        <v>525</v>
+        <v>514</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>263</v>
+        <v>165</v>
       </c>
       <c r="F50" s="10" t="s">
         <v>395</v>
@@ -6570,19 +6582,19 @@
         <v>134</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
       <c r="I50" s="10" t="s">
         <v>516</v>
       </c>
       <c r="J50" s="10" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="L50" s="10" t="s">
-        <v>529</v>
+        <v>503</v>
       </c>
       <c r="M50" s="10" t="s">
         <v>519</v>
@@ -6600,18 +6612,18 @@
         <v>117</v>
       </c>
       <c r="R50" s="10" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="S50" s="11" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="T50" s="10" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>404</v>
@@ -6632,19 +6644,19 @@
         <v>134</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
       <c r="J51" s="10" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="K51" s="10" t="s">
         <v>528</v>
       </c>
       <c r="L51" s="10" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="M51" s="10" t="s">
         <v>519</v>
@@ -6656,22 +6668,24 @@
         <v>520</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>538</v>
+        <v>521</v>
       </c>
       <c r="Q51" s="10" t="s">
-        <v>539</v>
+        <v>117</v>
       </c>
       <c r="R51" s="10" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="S51" s="11" t="s">
-        <v>541</v>
-      </c>
-      <c r="T51" s="10"/>
+        <v>531</v>
+      </c>
+      <c r="T51" s="10" t="s">
+        <v>532</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
-        <v>542</v>
+        <v>533</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>404</v>
@@ -6692,48 +6706,46 @@
         <v>134</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>543</v>
+        <v>534</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>516</v>
+        <v>535</v>
       </c>
       <c r="J52" s="10" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="K52" s="10" t="s">
         <v>528</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="M52" s="10" t="s">
-        <v>546</v>
+        <v>519</v>
       </c>
       <c r="N52" s="10" t="s">
         <v>12</v>
       </c>
       <c r="O52" s="10" t="s">
-        <v>547</v>
+        <v>520</v>
       </c>
       <c r="P52" s="10" t="s">
         <v>538</v>
       </c>
       <c r="Q52" s="10" t="s">
-        <v>117</v>
+        <v>539</v>
       </c>
       <c r="R52" s="10" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="S52" s="11" t="s">
-        <v>549</v>
-      </c>
-      <c r="T52" s="10" t="s">
-        <v>550</v>
-      </c>
+        <v>541</v>
+      </c>
+      <c r="T52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="s">
-        <v>551</v>
+        <v>542</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>404</v>
@@ -6748,52 +6760,54 @@
         <v>263</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>90</v>
+        <v>395</v>
       </c>
       <c r="G53" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>552</v>
+        <v>543</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>516</v>
       </c>
       <c r="J53" s="10" t="s">
-        <v>553</v>
+        <v>544</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="L53" s="10" t="s">
-        <v>420</v>
+        <v>545</v>
       </c>
       <c r="M53" s="10" t="s">
-        <v>519</v>
+        <v>546</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
       <c r="Q53" s="10" t="s">
         <v>117</v>
       </c>
       <c r="R53" s="10" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="S53" s="11" t="s">
-        <v>556</v>
-      </c>
-      <c r="T53" s="10"/>
+        <v>549</v>
+      </c>
+      <c r="T53" s="10" t="s">
+        <v>550</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>404</v>
@@ -6808,132 +6822,132 @@
         <v>263</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>217</v>
+        <v>90</v>
       </c>
       <c r="G54" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="H54" s="10" t="inlineStr">
+      <c r="H54" s="10" t="s">
+        <v>552</v>
+      </c>
+      <c r="I54" s="10" t="s">
+        <v>516</v>
+      </c>
+      <c r="J54" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="K54" s="10" t="s">
+        <v>493</v>
+      </c>
+      <c r="L54" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="M54" s="10" t="s">
+        <v>519</v>
+      </c>
+      <c r="N54" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="O54" s="10" t="s">
+        <v>554</v>
+      </c>
+      <c r="P54" s="10" t="s">
+        <v>521</v>
+      </c>
+      <c r="Q54" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="R54" s="10" t="s">
+        <v>555</v>
+      </c>
+      <c r="S54" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="T54" s="10"/>
+    </row>
+    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="s">
+        <v>557</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Formal pre-court diversion</t>
         </is>
       </c>
-      <c r="I54" s="10" t="inlineStr">
+      <c r="I55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Effect on reoffending and violence</t>
         </is>
       </c>
-      <c r="J54" s="10" t="inlineStr">
+      <c r="J55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">−14% reoffending (moderate confidence, 35 studies); −25% violence (low confidence, 5 studies); UK average cost £1,426 per child</t>
         </is>
       </c>
-      <c r="K54" s="10" t="inlineStr">
+      <c r="K55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Effective, cost unclear</t>
         </is>
       </c>
-      <c r="L54" s="10" t="s">
+      <c r="L55" s="10" t="s">
         <v>561</v>
       </c>
-      <c r="M54" s="10" t="s">
+      <c r="M55" s="10" t="s">
         <v>562</v>
       </c>
-      <c r="N54" s="10" t="s">
+      <c r="N55" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="O54" s="10" t="s">
+      <c r="O55" s="10" t="s">
         <v>520</v>
       </c>
-      <c r="P54" s="10" t="inlineStr">
+      <c r="P55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Mostly North America and Australia; UK costs</t>
         </is>
       </c>
-      <c r="Q54" s="10" t="inlineStr">
+      <c r="Q55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">not stated</t>
         </is>
       </c>
-      <c r="R54" s="10" t="inlineStr">
+      <c r="R55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Youth Endowment Fund Toolkit, Formal pre-court diversion</t>
         </is>
       </c>
-      <c r="S54" s="11" t="inlineStr">
+      <c r="S55" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">https://youthendowmentfund.org.uk/toolkit/formal-pre-court-diversion/</t>
         </is>
       </c>
-      <c r="T54" s="10" t="inlineStr">
+      <c r="T55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Replaces YEF's earlier pre-court diversion strand (−13% reoffending, high confidence, low cost). Informal pre-court diversion is now a separate strand.</t>
         </is>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10" t="s">
-        <v>566</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="F55" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G55" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>567</v>
-      </c>
-      <c r="I55" s="10" t="s">
-        <v>568</v>
-      </c>
-      <c r="J55" s="10" t="s">
-        <v>569</v>
-      </c>
-      <c r="K55" s="10" t="s">
-        <v>451</v>
-      </c>
-      <c r="L55" s="10" t="s">
-        <v>570</v>
-      </c>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="O55" s="10" t="s">
-        <v>571</v>
-      </c>
-      <c r="P55" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="Q55" s="10" t="s">
-        <v>454</v>
-      </c>
-      <c r="R55" s="10" t="s">
-        <v>572</v>
-      </c>
-      <c r="S55" s="11" t="s">
-        <v>573</v>
-      </c>
-      <c r="T55" s="10" t="s">
-        <v>574</v>
-      </c>
-    </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
-        <v>575</v>
+        <v>566</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>404</v>
@@ -6948,52 +6962,52 @@
         <v>165</v>
       </c>
       <c r="F56" s="10" t="s">
-        <v>217</v>
+        <v>76</v>
       </c>
       <c r="G56" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H56" s="10" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="K56" s="10" t="s">
         <v>451</v>
       </c>
       <c r="L56" s="10" t="s">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="M56" s="10"/>
       <c r="N56" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O56" s="10" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="P56" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q56" s="10" t="s">
-        <v>117</v>
+        <v>454</v>
       </c>
       <c r="R56" s="10" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="S56" s="11" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="T56" s="10" t="s">
-        <v>583</v>
+        <v>574</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
-        <v>584</v>
+        <v>575</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>404</v>
@@ -7005,119 +7019,117 @@
         <v>188</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>263</v>
+        <v>165</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>395</v>
+        <v>217</v>
       </c>
       <c r="G57" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>585</v>
+        <v>576</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>586</v>
+        <v>577</v>
       </c>
       <c r="J57" s="10" t="s">
-        <v>587</v>
+        <v>578</v>
       </c>
       <c r="K57" s="10" t="s">
-        <v>493</v>
+        <v>451</v>
       </c>
       <c r="L57" s="10" t="s">
-        <v>588</v>
-      </c>
-      <c r="M57" s="10" t="s">
-        <v>589</v>
-      </c>
+        <v>579</v>
+      </c>
+      <c r="M57" s="10"/>
       <c r="N57" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="Q57" s="10" t="s">
-        <v>591</v>
+        <v>117</v>
       </c>
       <c r="R57" s="10" t="s">
-        <v>592</v>
+        <v>581</v>
       </c>
       <c r="S57" s="11" t="s">
-        <v>593</v>
+        <v>582</v>
       </c>
       <c r="T57" s="10" t="s">
-        <v>594</v>
+        <v>583</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
-        <v>595</v>
+        <v>584</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>261</v>
+        <v>187</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>262</v>
+        <v>188</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>111</v>
+        <v>263</v>
       </c>
       <c r="F58" s="10" t="s">
-        <v>217</v>
+        <v>395</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>91</v>
+        <v>134</v>
       </c>
       <c r="H58" s="10" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>597</v>
+        <v>586</v>
       </c>
       <c r="J58" s="10" t="s">
-        <v>598</v>
+        <v>587</v>
       </c>
       <c r="K58" s="10" t="s">
-        <v>528</v>
+        <v>493</v>
       </c>
       <c r="L58" s="10" t="s">
-        <v>420</v>
+        <v>588</v>
       </c>
       <c r="M58" s="10" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="N58" s="10" t="s">
         <v>12</v>
       </c>
       <c r="O58" s="10" t="s">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="P58" s="10" t="s">
-        <v>601</v>
+        <v>70</v>
       </c>
       <c r="Q58" s="10" t="s">
-        <v>117</v>
+        <v>591</v>
       </c>
       <c r="R58" s="10" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
       <c r="S58" s="11" t="s">
-        <v>603</v>
+        <v>593</v>
       </c>
       <c r="T58" s="10" t="s">
-        <v>604</v>
+        <v>594</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>404</v>
@@ -7129,7 +7141,7 @@
         <v>262</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>216</v>
+        <v>111</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>217</v>
@@ -7138,181 +7150,181 @@
         <v>91</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="J59" s="10" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="K59" s="10" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="L59" s="10" t="s">
-        <v>609</v>
+        <v>420</v>
       </c>
       <c r="M59" s="10" t="s">
-        <v>610</v>
+        <v>599</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>81</v>
+        <v>601</v>
       </c>
       <c r="Q59" s="10" t="s">
-        <v>202</v>
+        <v>117</v>
       </c>
       <c r="R59" s="10" t="s">
-        <v>612</v>
+        <v>602</v>
       </c>
       <c r="S59" s="11" t="s">
-        <v>613</v>
+        <v>603</v>
       </c>
       <c r="T59" s="10" t="s">
-        <v>614</v>
+        <v>604</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
-        <v>615</v>
+        <v>605</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>187</v>
+        <v>261</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>188</v>
+        <v>262</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>263</v>
+        <v>216</v>
       </c>
       <c r="F60" s="10" t="s">
-        <v>395</v>
+        <v>217</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H60" s="10" t="s">
-        <v>616</v>
+        <v>606</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>501</v>
+        <v>607</v>
       </c>
       <c r="J60" s="10" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="L60" s="10" t="s">
-        <v>618</v>
+        <v>609</v>
       </c>
       <c r="M60" s="10" t="s">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="N60" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O60" s="10" t="s">
-        <v>620</v>
+        <v>611</v>
       </c>
       <c r="P60" s="10" t="s">
-        <v>268</v>
+        <v>81</v>
       </c>
       <c r="Q60" s="10" t="s">
-        <v>279</v>
+        <v>202</v>
       </c>
       <c r="R60" s="10" t="s">
-        <v>621</v>
+        <v>612</v>
       </c>
       <c r="S60" s="11" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="T60" s="10" t="s">
-        <v>623</v>
+        <v>614</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="10" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>261</v>
+        <v>187</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>262</v>
+        <v>188</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="F61" s="10" t="s">
-        <v>90</v>
+        <v>395</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="I61" s="10" t="s">
         <v>501</v>
       </c>
       <c r="J61" s="10" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="K61" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L61" s="10" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="M61" s="10" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="N61" s="10" t="s">
         <v>14</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>81</v>
+        <v>268</v>
       </c>
       <c r="Q61" s="10" t="s">
-        <v>202</v>
+        <v>279</v>
       </c>
       <c r="R61" s="10" t="s">
-        <v>630</v>
+        <v>621</v>
       </c>
       <c r="S61" s="11" t="s">
-        <v>631</v>
+        <v>622</v>
       </c>
       <c r="T61" s="10" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
-        <v>633</v>
+        <v>624</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>274</v>
@@ -7324,48 +7336,48 @@
         <v>91</v>
       </c>
       <c r="H62" s="10" t="s">
-        <v>634</v>
+        <v>625</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>406</v>
+        <v>501</v>
       </c>
       <c r="J62" s="10" t="s">
-        <v>635</v>
+        <v>626</v>
       </c>
       <c r="K62" s="10" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
       <c r="L62" s="10" t="s">
-        <v>420</v>
+        <v>627</v>
       </c>
       <c r="M62" s="10" t="s">
-        <v>636</v>
+        <v>628</v>
       </c>
       <c r="N62" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O62" s="10" t="s">
-        <v>637</v>
+        <v>629</v>
       </c>
       <c r="P62" s="10" t="s">
-        <v>638</v>
+        <v>81</v>
       </c>
       <c r="Q62" s="10" t="s">
-        <v>639</v>
+        <v>202</v>
       </c>
       <c r="R62" s="10" t="s">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="S62" s="11" t="s">
-        <v>641</v>
+        <v>631</v>
       </c>
       <c r="T62" s="10" t="s">
-        <v>642</v>
+        <v>632</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="10" t="s">
-        <v>643</v>
+        <v>633</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>404</v>
@@ -7380,54 +7392,54 @@
         <v>274</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>217</v>
+        <v>90</v>
       </c>
       <c r="G63" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>644</v>
+        <v>634</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>645</v>
+        <v>406</v>
       </c>
       <c r="J63" s="10" t="s">
-        <v>646</v>
+        <v>635</v>
       </c>
       <c r="K63" s="10" t="s">
-        <v>473</v>
+        <v>419</v>
       </c>
       <c r="L63" s="10" t="s">
-        <v>647</v>
+        <v>420</v>
       </c>
       <c r="M63" s="10" t="s">
-        <v>648</v>
+        <v>636</v>
       </c>
       <c r="N63" s="10" t="s">
         <v>12</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>649</v>
+        <v>637</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>81</v>
+        <v>638</v>
       </c>
       <c r="Q63" s="10" t="s">
-        <v>202</v>
+        <v>639</v>
       </c>
       <c r="R63" s="10" t="s">
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="S63" s="11" t="s">
-        <v>651</v>
+        <v>641</v>
       </c>
       <c r="T63" s="10" t="s">
-        <v>652</v>
+        <v>642</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
-        <v>653</v>
+        <v>643</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>404</v>
@@ -7442,54 +7454,54 @@
         <v>274</v>
       </c>
       <c r="F64" s="10" t="s">
-        <v>90</v>
+        <v>217</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>134</v>
+        <v>91</v>
       </c>
       <c r="H64" s="10" t="s">
-        <v>654</v>
+        <v>644</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>501</v>
+        <v>645</v>
       </c>
       <c r="J64" s="10" t="s">
-        <v>655</v>
+        <v>646</v>
       </c>
       <c r="K64" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L64" s="10" t="s">
-        <v>452</v>
+        <v>647</v>
       </c>
       <c r="M64" s="10" t="s">
-        <v>656</v>
+        <v>648</v>
       </c>
       <c r="N64" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O64" s="10" t="s">
-        <v>657</v>
+        <v>649</v>
       </c>
       <c r="P64" s="10" t="s">
         <v>81</v>
       </c>
       <c r="Q64" s="10" t="s">
-        <v>658</v>
+        <v>202</v>
       </c>
       <c r="R64" s="10" t="s">
-        <v>659</v>
+        <v>650</v>
       </c>
       <c r="S64" s="11" t="s">
-        <v>660</v>
+        <v>651</v>
       </c>
       <c r="T64" s="10" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
-        <v>662</v>
+        <v>653</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>404</v>
@@ -7500,56 +7512,58 @@
       <c r="D65" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E65" s="10"/>
+      <c r="E65" s="10" t="s">
+        <v>274</v>
+      </c>
       <c r="F65" s="10" t="s">
-        <v>395</v>
+        <v>90</v>
       </c>
       <c r="G65" s="10" t="s">
         <v>134</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>663</v>
+        <v>654</v>
       </c>
       <c r="I65" s="10" t="s">
         <v>501</v>
       </c>
       <c r="J65" s="10" t="s">
-        <v>664</v>
+        <v>655</v>
       </c>
       <c r="K65" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L65" s="10" t="s">
-        <v>545</v>
+        <v>452</v>
       </c>
       <c r="M65" s="10" t="s">
-        <v>665</v>
+        <v>656</v>
       </c>
       <c r="N65" s="10" t="s">
         <v>14</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>666</v>
+        <v>657</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="Q65" s="10" t="s">
-        <v>667</v>
+        <v>658</v>
       </c>
       <c r="R65" s="10" t="s">
-        <v>668</v>
+        <v>659</v>
       </c>
       <c r="S65" s="11" t="s">
-        <v>669</v>
+        <v>660</v>
       </c>
       <c r="T65" s="10" t="s">
-        <v>670</v>
+        <v>661</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
-        <v>671</v>
+        <v>662</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>404</v>
@@ -7568,48 +7582,48 @@
         <v>134</v>
       </c>
       <c r="H66" s="10" t="s">
-        <v>672</v>
+        <v>663</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>673</v>
+        <v>501</v>
       </c>
       <c r="J66" s="10" t="s">
-        <v>674</v>
+        <v>664</v>
       </c>
       <c r="K66" s="10" t="s">
-        <v>528</v>
+        <v>473</v>
       </c>
       <c r="L66" s="10" t="s">
-        <v>675</v>
+        <v>545</v>
       </c>
       <c r="M66" s="10" t="s">
-        <v>676</v>
+        <v>665</v>
       </c>
       <c r="N66" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O66" s="10" t="s">
-        <v>677</v>
+        <v>666</v>
       </c>
       <c r="P66" s="10" t="s">
         <v>70</v>
       </c>
       <c r="Q66" s="10" t="s">
-        <v>678</v>
+        <v>667</v>
       </c>
       <c r="R66" s="10" t="s">
-        <v>679</v>
+        <v>668</v>
       </c>
       <c r="S66" s="11" t="s">
-        <v>680</v>
+        <v>669</v>
       </c>
       <c r="T66" s="10" t="s">
-        <v>681</v>
+        <v>670</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>682</v>
+        <v>671</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>404</v>
@@ -7622,54 +7636,54 @@
       </c>
       <c r="E67" s="10"/>
       <c r="F67" s="10" t="s">
-        <v>323</v>
+        <v>395</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>65</v>
+        <v>134</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>683</v>
+        <v>672</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>684</v>
+        <v>673</v>
       </c>
       <c r="J67" s="10" t="s">
-        <v>685</v>
+        <v>674</v>
       </c>
       <c r="K67" s="10" t="s">
-        <v>473</v>
+        <v>528</v>
       </c>
       <c r="L67" s="10" t="s">
-        <v>686</v>
+        <v>675</v>
       </c>
       <c r="M67" s="10" t="s">
-        <v>687</v>
+        <v>676</v>
       </c>
       <c r="N67" s="10" t="s">
         <v>12</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>688</v>
+        <v>677</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>689</v>
+        <v>70</v>
       </c>
       <c r="Q67" s="10" t="s">
-        <v>279</v>
+        <v>678</v>
       </c>
       <c r="R67" s="10" t="s">
-        <v>690</v>
+        <v>679</v>
       </c>
       <c r="S67" s="11" t="s">
-        <v>691</v>
+        <v>680</v>
       </c>
       <c r="T67" s="10" t="s">
-        <v>692</v>
+        <v>681</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>693</v>
+        <v>682</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>404</v>
@@ -7680,100 +7694,98 @@
       <c r="D68" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E68" s="10" t="s">
-        <v>274</v>
-      </c>
+      <c r="E68" s="10"/>
       <c r="F68" s="10" t="s">
-        <v>176</v>
+        <v>323</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>65</v>
       </c>
       <c r="H68" s="10" t="s">
-        <v>694</v>
+        <v>683</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>695</v>
+        <v>684</v>
       </c>
       <c r="J68" s="10" t="s">
-        <v>696</v>
+        <v>685</v>
       </c>
       <c r="K68" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L68" s="10" t="s">
-        <v>697</v>
+        <v>686</v>
       </c>
       <c r="M68" s="10" t="s">
-        <v>698</v>
+        <v>687</v>
       </c>
       <c r="N68" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O68" s="10" t="s">
-        <v>699</v>
+        <v>688</v>
       </c>
       <c r="P68" s="10" t="s">
-        <v>81</v>
+        <v>689</v>
       </c>
       <c r="Q68" s="10" t="s">
-        <v>202</v>
+        <v>279</v>
       </c>
       <c r="R68" s="10" t="s">
-        <v>700</v>
+        <v>690</v>
       </c>
       <c r="S68" s="11" t="s">
-        <v>701</v>
+        <v>691</v>
       </c>
       <c r="T68" s="10" t="s">
-        <v>940</v>
+        <v>692</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
-        <v>702</v>
+        <v>693</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>274</v>
       </c>
       <c r="F69" s="10" t="s">
-        <v>76</v>
+        <v>176</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>703</v>
+        <v>694</v>
       </c>
       <c r="I69" s="10" t="s">
-        <v>501</v>
+        <v>695</v>
       </c>
       <c r="J69" s="10" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="K69" s="10" t="s">
         <v>473</v>
       </c>
       <c r="L69" s="10" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="M69" s="10" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="P69" s="10" t="s">
         <v>81</v>
@@ -7782,87 +7794,89 @@
         <v>202</v>
       </c>
       <c r="R69" s="10" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="S69" s="11" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="T69" s="10" t="s">
-        <v>710</v>
+        <v>940</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="10" t="s">
-        <v>711</v>
+        <v>702</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="E70" s="10"/>
+        <v>63</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>274</v>
+      </c>
       <c r="F70" s="10" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="G70" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H70" s="10" t="s">
-        <v>712</v>
+        <v>703</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>713</v>
+        <v>501</v>
       </c>
       <c r="J70" s="10" t="s">
-        <v>714</v>
+        <v>704</v>
       </c>
       <c r="K70" s="10" t="s">
-        <v>518</v>
+        <v>473</v>
       </c>
       <c r="L70" s="10" t="s">
-        <v>715</v>
+        <v>705</v>
       </c>
       <c r="M70" s="10" t="s">
-        <v>716</v>
+        <v>706</v>
       </c>
       <c r="N70" s="10" t="s">
         <v>12</v>
       </c>
       <c r="O70" s="10" t="s">
-        <v>717</v>
+        <v>707</v>
       </c>
       <c r="P70" s="10" t="s">
-        <v>718</v>
+        <v>81</v>
       </c>
       <c r="Q70" s="10" t="s">
-        <v>719</v>
+        <v>202</v>
       </c>
       <c r="R70" s="10" t="s">
-        <v>720</v>
+        <v>708</v>
       </c>
       <c r="S70" s="11" t="s">
-        <v>721</v>
+        <v>709</v>
       </c>
       <c r="T70" s="10" t="s">
-        <v>722</v>
+        <v>710</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="10" t="s">
-        <v>723</v>
+        <v>711</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E71" s="10"/>
       <c r="F71" s="10" t="s">
@@ -7872,48 +7886,48 @@
         <v>91</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>724</v>
+        <v>712</v>
       </c>
       <c r="I71" s="10" t="s">
-        <v>725</v>
+        <v>713</v>
       </c>
       <c r="J71" s="10" t="s">
-        <v>726</v>
+        <v>714</v>
       </c>
       <c r="K71" s="10" t="s">
-        <v>473</v>
+        <v>518</v>
       </c>
       <c r="L71" s="10" t="s">
-        <v>727</v>
+        <v>715</v>
       </c>
       <c r="M71" s="10" t="s">
-        <v>728</v>
+        <v>716</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>729</v>
+        <v>717</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>730</v>
+        <v>718</v>
       </c>
       <c r="Q71" s="10" t="s">
-        <v>731</v>
+        <v>719</v>
       </c>
       <c r="R71" s="10" t="s">
-        <v>732</v>
+        <v>720</v>
       </c>
       <c r="S71" s="11" t="s">
-        <v>733</v>
+        <v>721</v>
       </c>
       <c r="T71" s="10" t="s">
-        <v>734</v>
+        <v>722</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>735</v>
+        <v>723</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>404</v>
@@ -7932,182 +7946,182 @@
         <v>91</v>
       </c>
       <c r="H72" s="10" t="s">
-        <v>736</v>
+        <v>724</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>737</v>
+        <v>725</v>
       </c>
       <c r="J72" s="10" t="s">
-        <v>738</v>
+        <v>726</v>
       </c>
       <c r="K72" s="10" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
       <c r="L72" s="10" t="s">
-        <v>739</v>
+        <v>727</v>
       </c>
       <c r="M72" s="10" t="s">
-        <v>740</v>
+        <v>728</v>
       </c>
       <c r="N72" s="10" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O72" s="10" t="s">
-        <v>741</v>
+        <v>729</v>
       </c>
       <c r="P72" s="10" t="s">
-        <v>81</v>
+        <v>730</v>
       </c>
       <c r="Q72" s="10" t="s">
-        <v>247</v>
+        <v>731</v>
       </c>
       <c r="R72" s="10" t="s">
-        <v>742</v>
+        <v>732</v>
       </c>
       <c r="S72" s="11" t="s">
-        <v>743</v>
+        <v>733</v>
       </c>
       <c r="T72" s="10" t="s">
-        <v>744</v>
+        <v>734</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
-        <v>941</v>
+        <v>735</v>
       </c>
       <c r="B73" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>187</v>
+        <v>62</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>263</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="E73" s="10"/>
       <c r="F73" s="10" t="s">
-        <v>217</v>
+        <v>90</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>134</v>
+        <v>91</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>942</v>
+        <v>736</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>943</v>
+        <v>737</v>
       </c>
       <c r="J73" s="10" t="s">
-        <v>944</v>
+        <v>738</v>
       </c>
       <c r="K73" s="10" t="s">
-        <v>493</v>
+        <v>419</v>
       </c>
       <c r="L73" s="10" t="s">
-        <v>945</v>
+        <v>739</v>
       </c>
       <c r="M73" s="10" t="s">
-        <v>946</v>
+        <v>740</v>
       </c>
       <c r="N73" s="10" t="s">
         <v>14</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>947</v>
+        <v>741</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>948</v>
+        <v>81</v>
       </c>
       <c r="Q73" s="10" t="s">
-        <v>202</v>
+        <v>247</v>
       </c>
       <c r="R73" s="10" t="s">
-        <v>949</v>
+        <v>742</v>
       </c>
       <c r="S73" s="11" t="s">
-        <v>950</v>
+        <v>743</v>
       </c>
       <c r="T73" s="10" t="s">
-        <v>951</v>
+        <v>744</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10" t="s">
-        <v>954</v>
+        <v>941</v>
       </c>
       <c r="B74" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>122</v>
+        <v>263</v>
       </c>
       <c r="F74" s="10" t="s">
-        <v>153</v>
+        <v>217</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>91</v>
+        <v>134</v>
       </c>
       <c r="H74" s="10" t="s">
-        <v>955</v>
+        <v>942</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>956</v>
+        <v>943</v>
       </c>
       <c r="J74" s="10" t="s">
-        <v>957</v>
+        <v>944</v>
       </c>
       <c r="K74" s="10" t="s">
-        <v>528</v>
+        <v>493</v>
       </c>
       <c r="L74" s="10" t="s">
-        <v>503</v>
-      </c>
-      <c r="M74" s="10"/>
+        <v>945</v>
+      </c>
+      <c r="M74" s="10" t="s">
+        <v>946</v>
+      </c>
       <c r="N74" s="10" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="O74" s="10" t="s">
-        <v>958</v>
+        <v>947</v>
       </c>
       <c r="P74" s="10" t="s">
-        <v>81</v>
+        <v>948</v>
       </c>
       <c r="Q74" s="10" t="s">
         <v>202</v>
       </c>
       <c r="R74" s="10" t="s">
-        <v>959</v>
+        <v>949</v>
       </c>
       <c r="S74" s="11" t="s">
-        <v>960</v>
+        <v>950</v>
       </c>
       <c r="T74" s="10" t="s">
-        <v>961</v>
+        <v>951</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10" t="s">
-        <v>962</v>
+        <v>954</v>
       </c>
       <c r="B75" s="10" t="s">
         <v>404</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>165</v>
+        <v>122</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>153</v>
@@ -8116,96 +8130,104 @@
         <v>91</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>963</v>
+        <v>955</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>964</v>
+        <v>956</v>
       </c>
       <c r="J75" s="10" t="s">
-        <v>965</v>
+        <v>957</v>
       </c>
       <c r="K75" s="10" t="s">
-        <v>451</v>
-      </c>
-      <c r="L75" s="10"/>
+        <v>528</v>
+      </c>
+      <c r="L75" s="10" t="s">
+        <v>503</v>
+      </c>
       <c r="M75" s="10"/>
       <c r="N75" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>966</v>
+        <v>958</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>967</v>
+        <v>81</v>
       </c>
       <c r="Q75" s="10" t="s">
         <v>202</v>
       </c>
       <c r="R75" s="10" t="s">
-        <v>968</v>
+        <v>959</v>
       </c>
       <c r="S75" s="11" t="s">
-        <v>969</v>
+        <v>960</v>
       </c>
       <c r="T75" s="10" t="s">
-        <v>970</v>
+        <v>961</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10" t="s">
-        <v>745</v>
+        <v>962</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>746</v>
+        <v>404</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>62</v>
+        <v>163</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E76" s="10"/>
+        <v>164</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>165</v>
+      </c>
       <c r="F76" s="10" t="s">
-        <v>747</v>
-      </c>
-      <c r="G76" s="10"/>
+        <v>153</v>
+      </c>
+      <c r="G76" s="10" t="s">
+        <v>91</v>
+      </c>
       <c r="H76" s="10" t="s">
-        <v>748</v>
+        <v>963</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>749</v>
+        <v>964</v>
       </c>
       <c r="J76" s="10" t="s">
-        <v>750</v>
-      </c>
-      <c r="K76" s="10"/>
+        <v>965</v>
+      </c>
+      <c r="K76" s="10" t="s">
+        <v>451</v>
+      </c>
       <c r="L76" s="10"/>
       <c r="M76" s="10"/>
       <c r="N76" s="10" t="s">
         <v>10</v>
       </c>
       <c r="O76" s="10" t="s">
-        <v>751</v>
+        <v>966</v>
       </c>
       <c r="P76" s="10" t="s">
-        <v>96</v>
+        <v>967</v>
       </c>
       <c r="Q76" s="10" t="s">
-        <v>296</v>
+        <v>202</v>
       </c>
       <c r="R76" s="10" t="s">
-        <v>752</v>
+        <v>968</v>
       </c>
       <c r="S76" s="11" t="s">
-        <v>753</v>
+        <v>969</v>
       </c>
       <c r="T76" s="10" t="s">
-        <v>953</v>
+        <v>970</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10" t="s">
-        <v>755</v>
+        <v>745</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>746</v>
@@ -8222,13 +8244,13 @@
       </c>
       <c r="G77" s="10"/>
       <c r="H77" s="10" t="s">
-        <v>756</v>
+        <v>748</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>757</v>
+        <v>749</v>
       </c>
       <c r="J77" s="10" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
       <c r="K77" s="10"/>
       <c r="L77" s="10"/>
@@ -8237,27 +8259,27 @@
         <v>10</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>759</v>
+        <v>751</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q77" s="10" t="s">
-        <v>139</v>
+        <v>296</v>
       </c>
       <c r="R77" s="10" t="s">
-        <v>760</v>
+        <v>752</v>
       </c>
       <c r="S77" s="11" t="s">
-        <v>761</v>
+        <v>753</v>
       </c>
       <c r="T77" s="10" t="s">
-        <v>762</v>
+        <v>953</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10" t="s">
-        <v>763</v>
+        <v>755</v>
       </c>
       <c r="B78" s="10" t="s">
         <v>746</v>
@@ -8274,13 +8296,13 @@
       </c>
       <c r="G78" s="10"/>
       <c r="H78" s="10" t="s">
-        <v>764</v>
+        <v>756</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="J78" s="10" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="K78" s="10"/>
       <c r="L78" s="10"/>
@@ -8289,25 +8311,27 @@
         <v>10</v>
       </c>
       <c r="O78" s="10" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="P78" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q78" s="10" t="s">
-        <v>269</v>
+        <v>139</v>
       </c>
       <c r="R78" s="10" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="S78" s="11" t="s">
-        <v>768</v>
-      </c>
-      <c r="T78" s="10"/>
+        <v>761</v>
+      </c>
+      <c r="T78" s="10" t="s">
+        <v>762</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
       <c r="B79" s="10" t="s">
         <v>746</v>
@@ -8324,13 +8348,13 @@
       </c>
       <c r="G79" s="10"/>
       <c r="H79" s="10" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>771</v>
+        <v>749</v>
       </c>
       <c r="J79" s="10" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="K79" s="10"/>
       <c r="L79" s="10"/>
@@ -8339,27 +8363,25 @@
         <v>10</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q79" s="10" t="s">
         <v>269</v>
       </c>
       <c r="R79" s="10" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="S79" s="11" t="s">
-        <v>775</v>
-      </c>
-      <c r="T79" s="10" t="s">
-        <v>776</v>
-      </c>
+        <v>768</v>
+      </c>
+      <c r="T79" s="10"/>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>746</v>
@@ -8376,42 +8398,42 @@
       </c>
       <c r="G80" s="10"/>
       <c r="H80" s="10" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
       <c r="I80" s="10" t="s">
         <v>771</v>
       </c>
       <c r="J80" s="10" t="s">
-        <v>779</v>
+        <v>772</v>
       </c>
       <c r="K80" s="10"/>
       <c r="L80" s="10"/>
       <c r="M80" s="10"/>
       <c r="N80" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O80" s="10" t="s">
-        <v>780</v>
+        <v>773</v>
       </c>
       <c r="P80" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q80" s="10" t="s">
-        <v>781</v>
+        <v>269</v>
       </c>
       <c r="R80" s="10" t="s">
-        <v>782</v>
+        <v>774</v>
       </c>
       <c r="S80" s="11" t="s">
-        <v>783</v>
+        <v>775</v>
       </c>
       <c r="T80" s="10" t="s">
-        <v>784</v>
+        <v>776</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10" t="s">
-        <v>785</v>
+        <v>777</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>746</v>
@@ -8428,13 +8450,13 @@
       </c>
       <c r="G81" s="10"/>
       <c r="H81" s="10" t="s">
-        <v>786</v>
+        <v>778</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>787</v>
+        <v>771</v>
       </c>
       <c r="J81" s="10" t="s">
-        <v>788</v>
+        <v>779</v>
       </c>
       <c r="K81" s="10"/>
       <c r="L81" s="10"/>
@@ -8443,27 +8465,27 @@
         <v>12</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>789</v>
+        <v>780</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q81" s="10" t="s">
-        <v>790</v>
+        <v>781</v>
       </c>
       <c r="R81" s="10" t="s">
-        <v>791</v>
+        <v>782</v>
       </c>
       <c r="S81" s="11" t="s">
-        <v>792</v>
+        <v>783</v>
       </c>
       <c r="T81" s="10" t="s">
-        <v>793</v>
+        <v>784</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10" t="s">
-        <v>794</v>
+        <v>785</v>
       </c>
       <c r="B82" s="10" t="s">
         <v>746</v>
@@ -8480,96 +8502,94 @@
       </c>
       <c r="G82" s="10"/>
       <c r="H82" s="10" t="s">
-        <v>795</v>
+        <v>786</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>796</v>
+        <v>787</v>
       </c>
       <c r="J82" s="10" t="s">
-        <v>797</v>
+        <v>788</v>
       </c>
       <c r="K82" s="10"/>
       <c r="L82" s="10"/>
       <c r="M82" s="10"/>
       <c r="N82" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O82" s="10" t="s">
-        <v>798</v>
+        <v>789</v>
       </c>
       <c r="P82" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q82" s="10" t="s">
-        <v>658</v>
+        <v>790</v>
       </c>
       <c r="R82" s="10" t="s">
-        <v>799</v>
+        <v>791</v>
       </c>
       <c r="S82" s="11" t="s">
-        <v>800</v>
+        <v>792</v>
       </c>
       <c r="T82" s="10" t="s">
-        <v>801</v>
+        <v>793</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10" t="s">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>803</v>
+        <v>746</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E83" s="10"/>
       <c r="F83" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G83" s="10" t="s">
-        <v>91</v>
-      </c>
+        <v>747</v>
+      </c>
+      <c r="G83" s="10"/>
       <c r="H83" s="10" t="s">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>805</v>
+        <v>796</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>806</v>
+        <v>797</v>
       </c>
       <c r="K83" s="10"/>
       <c r="L83" s="10"/>
       <c r="M83" s="10"/>
       <c r="N83" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>807</v>
+        <v>798</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q83" s="10" t="s">
-        <v>312</v>
+        <v>658</v>
       </c>
       <c r="R83" s="10" t="s">
-        <v>808</v>
-      </c>
-      <c r="S83" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
-        </is>
-      </c>
-      <c r="T83" s="10"/>
+        <v>799</v>
+      </c>
+      <c r="S83" s="11" t="s">
+        <v>800</v>
+      </c>
+      <c r="T83" s="10" t="s">
+        <v>801</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10" t="s">
-        <v>810</v>
+        <v>802</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>803</v>
@@ -8582,19 +8602,19 @@
       </c>
       <c r="E84" s="10"/>
       <c r="F84" s="10" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H84" s="10" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="I84" s="10" t="s">
         <v>805</v>
       </c>
       <c r="J84" s="10" t="s">
-        <v>812</v>
+        <v>806</v>
       </c>
       <c r="K84" s="10"/>
       <c r="L84" s="10"/>
@@ -8612,95 +8632,97 @@
         <v>312</v>
       </c>
       <c r="R84" s="10" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="S84" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+          <t xml:space="preserve">https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england</t>
         </is>
       </c>
       <c r="T84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>63</v>
+        <v>234</v>
       </c>
       <c r="E85" s="10"/>
       <c r="F85" s="10" t="s">
-        <v>90</v>
+        <v>176</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>817</v>
+        <v>805</v>
       </c>
       <c r="J85" s="10" t="s">
-        <v>818</v>
+        <v>812</v>
       </c>
       <c r="K85" s="10"/>
       <c r="L85" s="10"/>
       <c r="M85" s="10"/>
       <c r="N85" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
       <c r="P85" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q85" s="10" t="s">
-        <v>269</v>
+        <v>312</v>
       </c>
       <c r="R85" s="10" t="s">
-        <v>820</v>
-      </c>
-      <c r="S85" s="11" t="s">
-        <v>821</v>
+        <v>813</v>
+      </c>
+      <c r="S85" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040</t>
+        </is>
       </c>
       <c r="T85" s="10"/>
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10" t="s">
-        <v>822</v>
+        <v>815</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>233</v>
+        <v>62</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>234</v>
+        <v>63</v>
       </c>
       <c r="E86" s="10"/>
       <c r="F86" s="10" t="s">
-        <v>176</v>
+        <v>90</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H86" s="10" t="s">
-        <v>823</v>
+        <v>816</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>824</v>
+        <v>817</v>
       </c>
       <c r="J86" s="10" t="s">
-        <v>825</v>
+        <v>818</v>
       </c>
       <c r="K86" s="10"/>
       <c r="L86" s="10"/>
@@ -8709,241 +8731,241 @@
         <v>10</v>
       </c>
       <c r="O86" s="10" t="s">
-        <v>826</v>
+        <v>819</v>
       </c>
       <c r="P86" s="10" t="s">
         <v>96</v>
       </c>
       <c r="Q86" s="10" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="R86" s="10" t="s">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="S86" s="11" t="s">
-        <v>828</v>
-      </c>
-      <c r="T86" s="10" t="s">
-        <v>829</v>
-      </c>
+        <v>821</v>
+      </c>
+      <c r="T86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10" t="s">
-        <v>830</v>
+        <v>822</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>163</v>
+        <v>233</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>111</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="E87" s="10"/>
       <c r="F87" s="10" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>831</v>
+        <v>823</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>832</v>
+        <v>824</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>833</v>
+        <v>825</v>
       </c>
       <c r="K87" s="10"/>
       <c r="L87" s="10"/>
       <c r="M87" s="10"/>
       <c r="N87" s="10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>834</v>
+        <v>826</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q87" s="10" t="s">
         <v>247</v>
       </c>
       <c r="R87" s="10" t="s">
-        <v>835</v>
+        <v>827</v>
       </c>
       <c r="S87" s="11" t="s">
-        <v>836</v>
+        <v>828</v>
       </c>
       <c r="T87" s="10" t="s">
-        <v>837</v>
+        <v>829</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="10" t="s">
-        <v>838</v>
+        <v>830</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>233</v>
+        <v>163</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="E88" s="10"/>
+        <v>164</v>
+      </c>
+      <c r="E88" s="10" t="s">
+        <v>111</v>
+      </c>
       <c r="F88" s="10" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="H88" s="10" t="s">
-        <v>388</v>
+        <v>831</v>
       </c>
       <c r="I88" s="10" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
       <c r="K88" s="10"/>
       <c r="L88" s="10"/>
       <c r="M88" s="10"/>
       <c r="N88" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O88" s="10" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="P88" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q88" s="10" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="R88" s="10" t="s">
-        <v>842</v>
+        <v>835</v>
       </c>
       <c r="S88" s="11" t="s">
-        <v>393</v>
-      </c>
-      <c r="T88" s="10"/>
+        <v>836</v>
+      </c>
+      <c r="T88" s="10" t="s">
+        <v>837</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="10" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>188</v>
+        <v>234</v>
       </c>
       <c r="E89" s="10"/>
       <c r="F89" s="10" t="s">
-        <v>76</v>
+        <v>176</v>
       </c>
       <c r="G89" s="10" t="s">
         <v>65</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>844</v>
+        <v>388</v>
       </c>
       <c r="I89" s="10" t="s">
-        <v>845</v>
+        <v>839</v>
       </c>
       <c r="J89" s="10" t="s">
-        <v>846</v>
+        <v>840</v>
       </c>
       <c r="K89" s="10"/>
       <c r="L89" s="10"/>
       <c r="M89" s="10"/>
       <c r="N89" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="Q89" s="10" t="s">
-        <v>848</v>
+        <v>193</v>
       </c>
       <c r="R89" s="10" t="s">
-        <v>849</v>
+        <v>842</v>
       </c>
       <c r="S89" s="11" t="s">
-        <v>850</v>
-      </c>
-      <c r="T89" s="10" t="s">
-        <v>851</v>
-      </c>
+        <v>393</v>
+      </c>
+      <c r="T89" s="10"/>
     </row>
     <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="10" t="s">
-        <v>852</v>
+        <v>843</v>
       </c>
       <c r="B90" s="10" t="s">
         <v>803</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>63</v>
+        <v>188</v>
       </c>
       <c r="E90" s="10"/>
       <c r="F90" s="10" t="s">
-        <v>176</v>
+        <v>76</v>
       </c>
       <c r="G90" s="10" t="s">
         <v>65</v>
       </c>
       <c r="H90" s="10" t="s">
-        <v>853</v>
+        <v>844</v>
       </c>
       <c r="I90" s="10" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="J90" s="10" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="K90" s="10"/>
       <c r="L90" s="10"/>
       <c r="M90" s="10"/>
       <c r="N90" s="10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O90" s="10" t="s">
-        <v>95</v>
+        <v>847</v>
       </c>
       <c r="P90" s="10" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="Q90" s="10" t="s">
-        <v>312</v>
+        <v>848</v>
       </c>
       <c r="R90" s="10" t="s">
-        <v>855</v>
+        <v>849</v>
       </c>
       <c r="S90" s="11" t="s">
-        <v>856</v>
-      </c>
-      <c r="T90" s="10"/>
+        <v>850</v>
+      </c>
+      <c r="T90" s="10" t="s">
+        <v>851</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="10" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="B91" s="10" t="s">
         <v>803</v>
@@ -8956,19 +8978,19 @@
       </c>
       <c r="E91" s="10"/>
       <c r="F91" s="10" t="s">
-        <v>64</v>
+        <v>176</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="I91" s="10" t="s">
-        <v>859</v>
+        <v>839</v>
       </c>
       <c r="J91" s="10" t="s">
-        <v>860</v>
+        <v>854</v>
       </c>
       <c r="K91" s="10"/>
       <c r="L91" s="10"/>
@@ -8977,26 +8999,78 @@
         <v>14</v>
       </c>
       <c r="O91" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="P91" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q91" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="R91" s="10" t="s">
+        <v>855</v>
+      </c>
+      <c r="S91" s="11" t="s">
+        <v>856</v>
+      </c>
+      <c r="T91" s="10"/>
+    </row>
+    <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="10" t="s">
+        <v>857</v>
+      </c>
+      <c r="B92" s="10" t="s">
+        <v>803</v>
+      </c>
+      <c r="C92" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E92" s="10"/>
+      <c r="F92" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G92" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H92" s="10" t="s">
+        <v>858</v>
+      </c>
+      <c r="I92" s="10" t="s">
+        <v>859</v>
+      </c>
+      <c r="J92" s="10" t="s">
+        <v>860</v>
+      </c>
+      <c r="K92" s="10"/>
+      <c r="L92" s="10"/>
+      <c r="M92" s="10"/>
+      <c r="N92" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="O92" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="P91" s="10" t="s">
+      <c r="P92" s="10" t="s">
         <v>861</v>
       </c>
-      <c r="Q91" s="10" t="s">
+      <c r="Q92" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="R91" s="10" t="s">
+      <c r="R92" s="10" t="s">
         <v>862</v>
       </c>
-      <c r="S91" s="11" t="s">
+      <c r="S92" s="11" t="s">
         <v>863</v>
       </c>
-      <c r="T91" s="10" t="s">
+      <c r="T92" s="10" t="s">
         <v>864</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T91"/>
+  <autoFilter ref="A1:T92"/>
   <hyperlinks>
     <hyperlink ref="S2" r:id="rId1" display="https://foundations.org.uk/our-work/publications/the-cost-of-late-intervention-eif-analysis-2016/"/>
     <hyperlink ref="S3" r:id="rId2" display="https://learning.nspcc.org.uk/research-resources/childrens-services-spending-reports"/>
@@ -9034,60 +9108,61 @@
     <hyperlink ref="S35" r:id="rId34" display="https://cls.ucl.ac.uk/wp-content/uploads/2017/02/Children-of-care-leavers-policy-briefing.pdf"/>
     <hyperlink ref="S36" r:id="rId35" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
     <hyperlink ref="S37" r:id="rId36" display="https://wrap.warwick.ac.uk/id/eprint/154072/"/>
-    <hyperlink ref="S38" r:id="rId37" display="https://doi.org/10.1017/S0033291718001940"/>
-    <hyperlink ref="S39" r:id="rId38" display="https://doi.org/10.1016/S2215-0366(25)00039-2"/>
-    <hyperlink ref="S40" r:id="rId39" display="https://doi.org/10.1111/add.13160"/>
-    <hyperlink ref="S41" r:id="rId40" display="https://doi.org/10.1111/add.16176"/>
-    <hyperlink ref="S42" r:id="rId41" display="https://doi.org/10.1111/jep.12799"/>
-    <hyperlink ref="S43" r:id="rId42" display="https://doi.org/10.1136/bmj.39126.699421.55"/>
-    <hyperlink ref="S44" r:id="rId43" display="https://link.springer.com/article/10.1186/1471-2458-11-803"/>
-    <hyperlink ref="S45" r:id="rId44" display="https://ifs.org.uk/news/sure-starts-wide-ranging-and-long-lasting-benefits-highlight-impact-integrated-early-years"/>
-    <hyperlink ref="S46" r:id="rId45" display="https://link.springer.com/article/10.1186/s12888-015-0700-x"/>
-    <hyperlink ref="S47" r:id="rId46" display="https://www.lse.ac.uk/business/consulting/assets/documents/commissioning-cost-effective-services-for-promotion-of-mental-health-and-wellbeing-and-prevention-of-mental-ill-health.pdf"/>
-    <hyperlink ref="S48" r:id="rId47" display="https://www.lse.ac.uk/business/consulting/assets/documents/commissioning-cost-effective-services-for-promotion-of-mental-health-and-wellbeing-and-prevention-of-mental-ill-health.pdf"/>
-    <hyperlink ref="S49" r:id="rId48" display="https://youthendowmentfund.org.uk/toolkit/social-skills-training/"/>
-    <hyperlink ref="S50" r:id="rId49" display="https://youthendowmentfund.org.uk/toolkit/cognitive-behavioural-therapy/"/>
-    <hyperlink ref="S51" r:id="rId50" display="https://youthendowmentfund.org.uk/toolkit/mentoring/"/>
-    <hyperlink ref="S52" r:id="rId51" display="https://youthendowmentfund.org.uk/toolkit/focused-deterrence/"/>
-    <hyperlink ref="S53" r:id="rId52" display="https://youthendowmentfund.org.uk/toolkit/trauma-specific-therapies/"/>
-    <hyperlink ref="S54" r:id="rId53" display="https://youthendowmentfund.org.uk/toolkit/formal-pre-court-diversion/"/>
-    <hyperlink ref="S55" r:id="rId54" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC6697182/"/>
-    <hyperlink ref="S56" r:id="rId55" display="https://doi.org/10.1111/jcpp.12743"/>
-    <hyperlink ref="S57" r:id="rId56" display="https://www.gov.uk/government/publications/violence-reduction-units-year-ending-march-2023-evaluation-report/violence-reduction-units-2022-to-2023"/>
-    <hyperlink ref="S58" r:id="rId57" display="https://doi.org/10.1056/NEJMoa1203241"/>
-    <hyperlink ref="S59" r:id="rId58" display="https://committees.parliament.uk/writtenevidence/72380/html/"/>
-    <hyperlink ref="S60" r:id="rId59" display="https://www.ukyouth.org/wp-content/uploads/2022/11/Economic-Value-of-Youth-Work-Full-Report.pdf"/>
-    <hyperlink ref="S61" r:id="rId60" display="https://eprints.lse.ac.uk/56773/"/>
-    <hyperlink ref="S62" r:id="rId61" display="https://doi.org/10.1192/bjp.bp.111.107888"/>
-    <hyperlink ref="S63" r:id="rId62" display="https://www.rand.org/pubs/research_briefs/RBA1271-1.html"/>
-    <hyperlink ref="S64" r:id="rId63" display="https://www.gov.uk/government/publications/alcohol-and-drug-prevention-treatment-and-recovery-why-invest/alcohol-and-drug-prevention-treatment-and-recovery-why-invest"/>
-    <hyperlink ref="S65" r:id="rId64" display="http://safelives.org.uk/research-policy-library/saving-lives-saving-money-report/"/>
-    <hyperlink ref="S66" r:id="rId65" display="https://safelives.org.uk/about-domestic-abuse/responding-to-perpetrators/"/>
-    <hyperlink ref="S67" r:id="rId66" display="https://assets.publishing.service.gov.uk/media/671a6fea603993b7a8f75db5/Housing_First_Cost_Benefit_Analysis_Report.pdf"/>
-    <hyperlink ref="S68" r:id="rId67" display="https://www.centreformentalhealth.org.uk/wp-content/uploads/2018/09/priorities.pdf"/>
-    <hyperlink ref="S69" r:id="rId68" display="https://assets.publishing.service.gov.uk/media/5fa2d5e2d3bf7f03b3ee4925/Pause_-_Sussex.pdf"/>
-    <hyperlink ref="S70" r:id="rId69" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10154457/"/>
-    <hyperlink ref="S71" r:id="rId70" display="https://pubmed.ncbi.nlm.nih.gov/28356325/"/>
-    <hyperlink ref="S72" r:id="rId71" display="https://www.health.org.uk/reports-and-analysis/analysis/investing-in-the-public-health-grant"/>
-    <hyperlink ref="S73" r:id="rId89" display="https://www.kurvekriegen.nrw.de/sites/default/files/2021-11/2016_03_Prognos_KNA_Managementsummary.pdf"/>
-    <hyperlink ref="S74" r:id="rId90" display="https://doi.org/10.1016/j.jsp.2022.04.006"/>
-    <hyperlink ref="S75" r:id="rId91" display="https://files.eric.ed.gov/fulltext/ED581531.pdf"/>
-    <hyperlink ref="S76" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
-    <hyperlink ref="S77" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
-    <hyperlink ref="S78" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
-    <hyperlink ref="S79" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
-    <hyperlink ref="S80" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
-    <hyperlink ref="S81" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
-    <hyperlink ref="S82" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
-    <hyperlink ref="S83" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
-    <hyperlink ref="S84" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
-    <hyperlink ref="S85" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
-    <hyperlink ref="S86" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
-    <hyperlink ref="S87" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
-    <hyperlink ref="S88" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
-    <hyperlink ref="S89" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
-    <hyperlink ref="S90" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
-    <hyperlink ref="S91" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
+    <hyperlink ref="S38" r:id="rId92" display="https://doi.org/10.1111/jcpp.12791"/>
+    <hyperlink ref="S39" r:id="rId37" display="https://doi.org/10.1017/S0033291718001940"/>
+    <hyperlink ref="S40" r:id="rId38" display="https://doi.org/10.1016/S2215-0366(25)00039-2"/>
+    <hyperlink ref="S41" r:id="rId39" display="https://doi.org/10.1111/add.13160"/>
+    <hyperlink ref="S42" r:id="rId40" display="https://doi.org/10.1111/add.16176"/>
+    <hyperlink ref="S43" r:id="rId41" display="https://doi.org/10.1111/jep.12799"/>
+    <hyperlink ref="S44" r:id="rId42" display="https://doi.org/10.1136/bmj.39126.699421.55"/>
+    <hyperlink ref="S45" r:id="rId43" display="https://link.springer.com/article/10.1186/1471-2458-11-803"/>
+    <hyperlink ref="S46" r:id="rId44" display="https://ifs.org.uk/news/sure-starts-wide-ranging-and-long-lasting-benefits-highlight-impact-integrated-early-years"/>
+    <hyperlink ref="S47" r:id="rId45" display="https://link.springer.com/article/10.1186/s12888-015-0700-x"/>
+    <hyperlink ref="S48" r:id="rId46" display="https://www.lse.ac.uk/business/consulting/assets/documents/commissioning-cost-effective-services-for-promotion-of-mental-health-and-wellbeing-and-prevention-of-mental-ill-health.pdf"/>
+    <hyperlink ref="S49" r:id="rId47" display="https://www.lse.ac.uk/business/consulting/assets/documents/commissioning-cost-effective-services-for-promotion-of-mental-health-and-wellbeing-and-prevention-of-mental-ill-health.pdf"/>
+    <hyperlink ref="S50" r:id="rId48" display="https://youthendowmentfund.org.uk/toolkit/social-skills-training/"/>
+    <hyperlink ref="S51" r:id="rId49" display="https://youthendowmentfund.org.uk/toolkit/cognitive-behavioural-therapy/"/>
+    <hyperlink ref="S52" r:id="rId50" display="https://youthendowmentfund.org.uk/toolkit/mentoring/"/>
+    <hyperlink ref="S53" r:id="rId51" display="https://youthendowmentfund.org.uk/toolkit/focused-deterrence/"/>
+    <hyperlink ref="S54" r:id="rId52" display="https://youthendowmentfund.org.uk/toolkit/trauma-specific-therapies/"/>
+    <hyperlink ref="S55" r:id="rId53" display="https://youthendowmentfund.org.uk/toolkit/formal-pre-court-diversion/"/>
+    <hyperlink ref="S56" r:id="rId54" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC6697182/"/>
+    <hyperlink ref="S57" r:id="rId55" display="https://doi.org/10.1111/jcpp.12743"/>
+    <hyperlink ref="S58" r:id="rId56" display="https://www.gov.uk/government/publications/violence-reduction-units-year-ending-march-2023-evaluation-report/violence-reduction-units-2022-to-2023"/>
+    <hyperlink ref="S59" r:id="rId57" display="https://doi.org/10.1056/NEJMoa1203241"/>
+    <hyperlink ref="S60" r:id="rId58" display="https://committees.parliament.uk/writtenevidence/72380/html/"/>
+    <hyperlink ref="S61" r:id="rId59" display="https://www.ukyouth.org/wp-content/uploads/2022/11/Economic-Value-of-Youth-Work-Full-Report.pdf"/>
+    <hyperlink ref="S62" r:id="rId60" display="https://eprints.lse.ac.uk/56773/"/>
+    <hyperlink ref="S63" r:id="rId61" display="https://doi.org/10.1192/bjp.bp.111.107888"/>
+    <hyperlink ref="S64" r:id="rId62" display="https://www.rand.org/pubs/research_briefs/RBA1271-1.html"/>
+    <hyperlink ref="S65" r:id="rId63" display="https://www.gov.uk/government/publications/alcohol-and-drug-prevention-treatment-and-recovery-why-invest/alcohol-and-drug-prevention-treatment-and-recovery-why-invest"/>
+    <hyperlink ref="S66" r:id="rId64" display="http://safelives.org.uk/research-policy-library/saving-lives-saving-money-report/"/>
+    <hyperlink ref="S67" r:id="rId65" display="https://safelives.org.uk/about-domestic-abuse/responding-to-perpetrators/"/>
+    <hyperlink ref="S68" r:id="rId66" display="https://assets.publishing.service.gov.uk/media/671a6fea603993b7a8f75db5/Housing_First_Cost_Benefit_Analysis_Report.pdf"/>
+    <hyperlink ref="S69" r:id="rId67" display="https://www.centreformentalhealth.org.uk/wp-content/uploads/2018/09/priorities.pdf"/>
+    <hyperlink ref="S70" r:id="rId68" display="https://assets.publishing.service.gov.uk/media/5fa2d5e2d3bf7f03b3ee4925/Pause_-_Sussex.pdf"/>
+    <hyperlink ref="S71" r:id="rId69" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10154457/"/>
+    <hyperlink ref="S72" r:id="rId70" display="https://pubmed.ncbi.nlm.nih.gov/28356325/"/>
+    <hyperlink ref="S73" r:id="rId71" display="https://www.health.org.uk/reports-and-analysis/analysis/investing-in-the-public-health-grant"/>
+    <hyperlink ref="S74" r:id="rId89" display="https://www.kurvekriegen.nrw.de/sites/default/files/2021-11/2016_03_Prognos_KNA_Managementsummary.pdf"/>
+    <hyperlink ref="S75" r:id="rId90" display="https://doi.org/10.1016/j.jsp.2022.04.006"/>
+    <hyperlink ref="S76" r:id="rId91" display="https://files.eric.ed.gov/fulltext/ED581531.pdf"/>
+    <hyperlink ref="S77" r:id="rId72" display="https://www.ohe.org/wp-content/uploads/2020/08/The_Green_Book.pdf"/>
+    <hyperlink ref="S78" r:id="rId73" display="https://assets.publishing.service.gov.uk/media/60fa9169d3bf7f0448719daf/Wellbeing_guidance_for_appraisal_-_supplementary_Green_Book_guidance.pdf"/>
+    <hyperlink ref="S79" r:id="rId74" display="https://www.nice.org.uk/news/articles/changes-to-nice-s-cost-effectiveness-thresholds-confirmed"/>
+    <hyperlink ref="S80" r:id="rId75" display="https://assets.publishing.service.gov.uk/media/698488ab2df808759a7bd70f/Green_Book_supplementary_guidance_-_discounting.pdf"/>
+    <hyperlink ref="S81" r:id="rId76" display="https://assets.publishing.service.gov.uk/media/6a43915e7ac6fd9c6a94abbe/Findings_and_Recommendations_-_Green_Book_Discount_Rate_Review.pdf"/>
+    <hyperlink ref="S82" r:id="rId77" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC13223565"/>
+    <hyperlink ref="S83" r:id="rId78" display="https://assets.publishing.service.gov.uk/government/uploads/system/uploads/attachment_data/file/753688/Prevention_is_better_than_cure_5-11.pdf"/>
+    <hyperlink ref="S84" r:id="rId79" display="https://www.health.org.uk/reports-and-analysis/reports/health-in-2040-projected-patterns-of-illness-in-england"/>
+    <hyperlink ref="S85" r:id="rId80" display="https://www.health.org.uk/media-office/press-releases/700000-more-workers-are-projected-to-be-living-with-major-illness-by-2040"/>
+    <hyperlink ref="S86" r:id="rId81" display="https://assets.publishing.service.gov.uk/media/6a4cb4c74889d85e75ab40e0/E03599617_OBR_FRS_2026_Accessible.pdf"/>
+    <hyperlink ref="S87" r:id="rId82" display="https://obr.uk/frs/fiscal-risks-and-sustainability-july-2025/"/>
+    <hyperlink ref="S88" r:id="rId83" display="https://ifs.org.uk/publications/schools-and-colleges-2025-spending-review"/>
+    <hyperlink ref="S89" r:id="rId84" display="https://ippr-org.files.svdcdn.com/production/Downloads/Our_greatest_asset_Sept24.pdf"/>
+    <hyperlink ref="S90" r:id="rId85" display="https://youthendowmentfund.org.uk/reports/beyond-the-headlines-2026/"/>
+    <hyperlink ref="S91" r:id="rId86" display="https://cpag.org.uk/news/cost-child-poverty-2023"/>
+    <hyperlink ref="S92" r:id="rId87" display="https://www.thelancet.com/journals/lanpub/article/PIIS2468-2667(19)30145-8/fulltext"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>